<commit_message>
Extract punch data for employees 38, 39, 40 (folder 3 batch)
Covers 40 of ~80 uploaded images now (folders 3 and 4 complete).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PeUzxoX8Admt6BxLMC3Cdz
</commit_message>
<xml_diff>
--- a/output/timesheet.xlsx
+++ b/output/timesheet.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G78"/>
+  <dimension ref="A1:G157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2602,6 +2602,2179 @@
         </is>
       </c>
     </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>Employee 38</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="D79" s="2" t="n"/>
+      <c r="E79" s="4" t="n">
+        <v>0.2527777777777778</v>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151731.jpg</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>single punch only</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>Employee 38</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="n">
+        <v>46264</v>
+      </c>
+      <c r="D80" s="4" t="n">
+        <v>0.75625</v>
+      </c>
+      <c r="E80" s="4" t="n">
+        <v>0.2965277777777778</v>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151731.jpg</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>Employee 38</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="n">
+        <v>46263</v>
+      </c>
+      <c r="D81" s="4" t="n">
+        <v>0.7326388888888888</v>
+      </c>
+      <c r="E81" s="4" t="n">
+        <v>0.2965277777777778</v>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151731.jpg</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>Employee 38</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="n">
+        <v>46261</v>
+      </c>
+      <c r="D82" s="4" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E82" s="4" t="n">
+        <v>0.2666666666666667</v>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151731.jpg</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>Employee 38</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="n">
+        <v>46260</v>
+      </c>
+      <c r="D83" s="4" t="n">
+        <v>0.7534722222222222</v>
+      </c>
+      <c r="E83" s="4" t="n">
+        <v>0.3243055555555556</v>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151737.jpg</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>extra punch: 17:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>Employee 38</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="n">
+        <v>46259</v>
+      </c>
+      <c r="D84" s="4" t="n">
+        <v>0.7548611111111111</v>
+      </c>
+      <c r="E84" s="4" t="n">
+        <v>0.2763888888888889</v>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151737.jpg</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>Employee 38</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="n">
+        <v>46258</v>
+      </c>
+      <c r="D85" s="4" t="n">
+        <v>0.7388888888888889</v>
+      </c>
+      <c r="E85" s="4" t="n">
+        <v>0.3263888888888889</v>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151737.jpg</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>Employee 38</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="n">
+        <v>46257</v>
+      </c>
+      <c r="D86" s="4" t="n">
+        <v>0.7493055555555556</v>
+      </c>
+      <c r="E86" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151737.jpg</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>Employee 38</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="n">
+        <v>46256</v>
+      </c>
+      <c r="D87" s="4" t="n">
+        <v>0.7243055555555555</v>
+      </c>
+      <c r="E87" s="4" t="n">
+        <v>0.2069444444444444</v>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151742.jpg</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>Employee 38</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="n">
+        <v>46254</v>
+      </c>
+      <c r="D88" s="2" t="n"/>
+      <c r="E88" s="4" t="n">
+        <v>0.3576388888888889</v>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151742.jpg</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>single punch only</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>Employee 38</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="n">
+        <v>46253</v>
+      </c>
+      <c r="D89" s="4" t="n">
+        <v>0.7173611111111111</v>
+      </c>
+      <c r="E89" s="4" t="n">
+        <v>0.475</v>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151742.jpg</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>Employee 38</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="n">
+        <v>46252</v>
+      </c>
+      <c r="D90" s="4" t="n">
+        <v>0.7583333333333333</v>
+      </c>
+      <c r="E90" s="4" t="n">
+        <v>0.3083333333333333</v>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151742.jpg</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>Employee 38</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="n">
+        <v>46251</v>
+      </c>
+      <c r="D91" s="4" t="n">
+        <v>0.7680555555555556</v>
+      </c>
+      <c r="E91" s="4" t="n">
+        <v>0.3979166666666666</v>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151746.jpg</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>Employee 38</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="n">
+        <v>46250</v>
+      </c>
+      <c r="D92" s="4" t="n">
+        <v>0.7722222222222223</v>
+      </c>
+      <c r="E92" s="4" t="n">
+        <v>0.325</v>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151746.jpg</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>Employee 38</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="D93" s="4" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E93" s="4" t="n">
+        <v>0.2354166666666667</v>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151746.jpg</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>Employee 38</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="n">
+        <v>46247</v>
+      </c>
+      <c r="D94" s="2" t="n"/>
+      <c r="E94" s="4" t="n">
+        <v>0.3347222222222222</v>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151746.jpg</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>single punch only</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>Employee 38</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="n">
+        <v>46246</v>
+      </c>
+      <c r="D95" s="2" t="n"/>
+      <c r="E95" s="4" t="n">
+        <v>0.2986111111111111</v>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151751.jpg</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>single punch only</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>Employee 38</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="n">
+        <v>46245</v>
+      </c>
+      <c r="D96" s="2" t="n"/>
+      <c r="E96" s="4" t="n">
+        <v>0.3118055555555556</v>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151751.jpg</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>single punch only</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>Employee 38</t>
+        </is>
+      </c>
+      <c r="C97" s="3" t="n">
+        <v>46244</v>
+      </c>
+      <c r="D97" s="4" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E97" s="4" t="n">
+        <v>0.2263888888888889</v>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151751.jpg</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>Employee 38</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="n">
+        <v>46243</v>
+      </c>
+      <c r="D98" s="4" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E98" s="4" t="n">
+        <v>0.2798611111111111</v>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151751.jpg</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>Employee 38</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="n">
+        <v>46242</v>
+      </c>
+      <c r="D99" s="4" t="n">
+        <v>0.7604166666666666</v>
+      </c>
+      <c r="E99" s="4" t="n">
+        <v>0.3055555555555556</v>
+      </c>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151757.jpg</t>
+        </is>
+      </c>
+      <c r="G99" s="2" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>Employee 38</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="n">
+        <v>46240</v>
+      </c>
+      <c r="D100" s="4" t="n">
+        <v>0.7590277777777777</v>
+      </c>
+      <c r="E100" s="4" t="n">
+        <v>0.30625</v>
+      </c>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151757.jpg</t>
+        </is>
+      </c>
+      <c r="G100" s="2" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>Employee 38</t>
+        </is>
+      </c>
+      <c r="C101" s="3" t="n">
+        <v>46239</v>
+      </c>
+      <c r="D101" s="4" t="n">
+        <v>0.7715277777777778</v>
+      </c>
+      <c r="E101" s="4" t="n">
+        <v>0.3222222222222222</v>
+      </c>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151757.jpg</t>
+        </is>
+      </c>
+      <c r="G101" s="2" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>Employee 38</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="n">
+        <v>46238</v>
+      </c>
+      <c r="D102" s="4" t="n">
+        <v>0.7166666666666667</v>
+      </c>
+      <c r="E102" s="4" t="n">
+        <v>0.2763888888888889</v>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151757.jpg</t>
+        </is>
+      </c>
+      <c r="G102" s="2" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>Employee 38</t>
+        </is>
+      </c>
+      <c r="C103" s="3" t="n">
+        <v>46237</v>
+      </c>
+      <c r="D103" s="4" t="n">
+        <v>0.7159722222222222</v>
+      </c>
+      <c r="E103" s="4" t="n">
+        <v>0.3034722222222222</v>
+      </c>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151759.jpg</t>
+        </is>
+      </c>
+      <c r="G103" s="2" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>Employee 38</t>
+        </is>
+      </c>
+      <c r="C104" s="3" t="n">
+        <v>46236</v>
+      </c>
+      <c r="D104" s="4" t="n">
+        <v>0.7430555555555556</v>
+      </c>
+      <c r="E104" s="4" t="n">
+        <v>0.2958333333333333</v>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151759.jpg</t>
+        </is>
+      </c>
+      <c r="G104" s="2" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>Employee 38</t>
+        </is>
+      </c>
+      <c r="C105" s="3" t="n">
+        <v>46235</v>
+      </c>
+      <c r="D105" s="4" t="n">
+        <v>0.7458333333333333</v>
+      </c>
+      <c r="E105" s="4" t="n">
+        <v>0.2381944444444444</v>
+      </c>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151759.jpg</t>
+        </is>
+      </c>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>last day of month; final record</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>Employee 39</t>
+        </is>
+      </c>
+      <c r="C106" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="D106" s="2" t="n"/>
+      <c r="E106" s="4" t="n">
+        <v>0.2777777777777778</v>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151809.jpg</t>
+        </is>
+      </c>
+      <c r="G106" s="2" t="inlineStr">
+        <is>
+          <t>single punch only</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>Employee 39</t>
+        </is>
+      </c>
+      <c r="C107" s="3" t="n">
+        <v>46264</v>
+      </c>
+      <c r="D107" s="4" t="n">
+        <v>0.7541666666666667</v>
+      </c>
+      <c r="E107" s="4" t="n">
+        <v>0.2590277777777778</v>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151809.jpg</t>
+        </is>
+      </c>
+      <c r="G107" s="2" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>Employee 39</t>
+        </is>
+      </c>
+      <c r="C108" s="3" t="n">
+        <v>46263</v>
+      </c>
+      <c r="D108" s="4" t="n">
+        <v>0.7458333333333333</v>
+      </c>
+      <c r="E108" s="4" t="n">
+        <v>0.2569444444444444</v>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151809.jpg</t>
+        </is>
+      </c>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>extra punch: 17:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>Employee 39</t>
+        </is>
+      </c>
+      <c r="C109" s="3" t="n">
+        <v>46262</v>
+      </c>
+      <c r="D109" s="2" t="n"/>
+      <c r="E109" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151809.jpg</t>
+        </is>
+      </c>
+      <c r="G109" s="2" t="inlineStr">
+        <is>
+          <t>single punch only</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>Employee 39</t>
+        </is>
+      </c>
+      <c r="C110" s="3" t="n">
+        <v>46261</v>
+      </c>
+      <c r="D110" s="4" t="n">
+        <v>0.7944444444444444</v>
+      </c>
+      <c r="E110" s="4" t="n">
+        <v>0.2493055555555556</v>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151819.jpg</t>
+        </is>
+      </c>
+      <c r="G110" s="2" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>Employee 39</t>
+        </is>
+      </c>
+      <c r="C111" s="3" t="n">
+        <v>46260</v>
+      </c>
+      <c r="D111" s="4" t="n">
+        <v>0.7555555555555555</v>
+      </c>
+      <c r="E111" s="4" t="n">
+        <v>0.2479166666666667</v>
+      </c>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151819.jpg</t>
+        </is>
+      </c>
+      <c r="G111" s="2" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>Employee 39</t>
+        </is>
+      </c>
+      <c r="C112" s="3" t="n">
+        <v>46259</v>
+      </c>
+      <c r="D112" s="4" t="n">
+        <v>0.7597222222222222</v>
+      </c>
+      <c r="E112" s="4" t="n">
+        <v>0.2375</v>
+      </c>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151819.jpg</t>
+        </is>
+      </c>
+      <c r="G112" s="2" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>Employee 39</t>
+        </is>
+      </c>
+      <c r="C113" s="3" t="n">
+        <v>46258</v>
+      </c>
+      <c r="D113" s="4" t="n">
+        <v>0.7506944444444444</v>
+      </c>
+      <c r="E113" s="4" t="n">
+        <v>0.2375</v>
+      </c>
+      <c r="F113" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151819.jpg</t>
+        </is>
+      </c>
+      <c r="G113" s="2" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>Employee 39</t>
+        </is>
+      </c>
+      <c r="C114" s="3" t="n">
+        <v>46257</v>
+      </c>
+      <c r="D114" s="4" t="n">
+        <v>0.7618055555555555</v>
+      </c>
+      <c r="E114" s="4" t="n">
+        <v>0.2479166666666667</v>
+      </c>
+      <c r="F114" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151826.jpg</t>
+        </is>
+      </c>
+      <c r="G114" s="2" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>Employee 39</t>
+        </is>
+      </c>
+      <c r="C115" s="3" t="n">
+        <v>46256</v>
+      </c>
+      <c r="D115" s="2" t="n"/>
+      <c r="E115" s="4" t="n">
+        <v>0.2875</v>
+      </c>
+      <c r="F115" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151826.jpg</t>
+        </is>
+      </c>
+      <c r="G115" s="2" t="inlineStr">
+        <is>
+          <t>single punch only</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>Employee 39</t>
+        </is>
+      </c>
+      <c r="C116" s="3" t="n">
+        <v>46254</v>
+      </c>
+      <c r="D116" s="4" t="n">
+        <v>0.7243055555555555</v>
+      </c>
+      <c r="E116" s="4" t="n">
+        <v>0.2472222222222222</v>
+      </c>
+      <c r="F116" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151826.jpg</t>
+        </is>
+      </c>
+      <c r="G116" s="2" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>Employee 39</t>
+        </is>
+      </c>
+      <c r="C117" s="3" t="n">
+        <v>46253</v>
+      </c>
+      <c r="D117" s="4" t="n">
+        <v>0.7416666666666667</v>
+      </c>
+      <c r="E117" s="4" t="n">
+        <v>0.2395833333333333</v>
+      </c>
+      <c r="F117" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151826.jpg</t>
+        </is>
+      </c>
+      <c r="G117" s="2" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>Employee 39</t>
+        </is>
+      </c>
+      <c r="C118" s="3" t="n">
+        <v>46252</v>
+      </c>
+      <c r="D118" s="4" t="n">
+        <v>0.7416666666666667</v>
+      </c>
+      <c r="E118" s="4" t="n">
+        <v>0.2916666666666667</v>
+      </c>
+      <c r="F118" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151831.jpg</t>
+        </is>
+      </c>
+      <c r="G118" s="2" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B119" s="2" t="inlineStr">
+        <is>
+          <t>Employee 39</t>
+        </is>
+      </c>
+      <c r="C119" s="3" t="n">
+        <v>46251</v>
+      </c>
+      <c r="D119" s="4" t="n">
+        <v>0.7326388888888888</v>
+      </c>
+      <c r="E119" s="4" t="n">
+        <v>0.3416666666666667</v>
+      </c>
+      <c r="F119" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151831.jpg</t>
+        </is>
+      </c>
+      <c r="G119" s="2" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>Employee 39</t>
+        </is>
+      </c>
+      <c r="C120" s="3" t="n">
+        <v>46250</v>
+      </c>
+      <c r="D120" s="4" t="n">
+        <v>0.7381944444444445</v>
+      </c>
+      <c r="E120" s="4" t="n">
+        <v>0.2409722222222222</v>
+      </c>
+      <c r="F120" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151831.jpg</t>
+        </is>
+      </c>
+      <c r="G120" s="2" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>Employee 39</t>
+        </is>
+      </c>
+      <c r="C121" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="D121" s="4" t="n">
+        <v>0.7611111111111111</v>
+      </c>
+      <c r="E121" s="4" t="n">
+        <v>0.2354166666666667</v>
+      </c>
+      <c r="F121" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151831.jpg</t>
+        </is>
+      </c>
+      <c r="G121" s="2" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>Employee 39</t>
+        </is>
+      </c>
+      <c r="C122" s="3" t="n">
+        <v>46247</v>
+      </c>
+      <c r="D122" s="2" t="n"/>
+      <c r="E122" s="4" t="n">
+        <v>0.4402777777777778</v>
+      </c>
+      <c r="F122" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151837.jpg</t>
+        </is>
+      </c>
+      <c r="G122" s="2" t="inlineStr">
+        <is>
+          <t>single punch only</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>Employee 39</t>
+        </is>
+      </c>
+      <c r="C123" s="3" t="n">
+        <v>46246</v>
+      </c>
+      <c r="D123" s="4" t="n">
+        <v>0.7423611111111111</v>
+      </c>
+      <c r="E123" s="4" t="n">
+        <v>0.2284722222222222</v>
+      </c>
+      <c r="F123" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151837.jpg</t>
+        </is>
+      </c>
+      <c r="G123" s="2" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>Employee 39</t>
+        </is>
+      </c>
+      <c r="C124" s="3" t="n">
+        <v>46245</v>
+      </c>
+      <c r="D124" s="4" t="n">
+        <v>0.7375</v>
+      </c>
+      <c r="E124" s="4" t="n">
+        <v>0.2375</v>
+      </c>
+      <c r="F124" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151837.jpg</t>
+        </is>
+      </c>
+      <c r="G124" s="2" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>Employee 39</t>
+        </is>
+      </c>
+      <c r="C125" s="3" t="n">
+        <v>46244</v>
+      </c>
+      <c r="D125" s="4" t="n">
+        <v>0.7611111111111111</v>
+      </c>
+      <c r="E125" s="4" t="n">
+        <v>0.2256944444444444</v>
+      </c>
+      <c r="F125" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151837.jpg</t>
+        </is>
+      </c>
+      <c r="G125" s="2" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>Employee 39</t>
+        </is>
+      </c>
+      <c r="C126" s="3" t="n">
+        <v>46243</v>
+      </c>
+      <c r="D126" s="4" t="n">
+        <v>0.725</v>
+      </c>
+      <c r="E126" s="4" t="n">
+        <v>0.2395833333333333</v>
+      </c>
+      <c r="F126" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151844.jpg</t>
+        </is>
+      </c>
+      <c r="G126" s="2" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>Employee 39</t>
+        </is>
+      </c>
+      <c r="C127" s="3" t="n">
+        <v>46242</v>
+      </c>
+      <c r="D127" s="4" t="n">
+        <v>0.7618055555555555</v>
+      </c>
+      <c r="E127" s="4" t="n">
+        <v>0.2201388888888889</v>
+      </c>
+      <c r="F127" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151844.jpg</t>
+        </is>
+      </c>
+      <c r="G127" s="2" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>Employee 39</t>
+        </is>
+      </c>
+      <c r="C128" s="3" t="n">
+        <v>46240</v>
+      </c>
+      <c r="D128" s="4" t="n">
+        <v>0.7625</v>
+      </c>
+      <c r="E128" s="4" t="n">
+        <v>0.2409722222222222</v>
+      </c>
+      <c r="F128" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151844.jpg</t>
+        </is>
+      </c>
+      <c r="G128" s="2" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B129" s="2" t="inlineStr">
+        <is>
+          <t>Employee 39</t>
+        </is>
+      </c>
+      <c r="C129" s="3" t="n">
+        <v>46239</v>
+      </c>
+      <c r="D129" s="4" t="n">
+        <v>0.7722222222222223</v>
+      </c>
+      <c r="E129" s="4" t="n">
+        <v>0.4743055555555555</v>
+      </c>
+      <c r="F129" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151844.jpg</t>
+        </is>
+      </c>
+      <c r="G129" s="2" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>Employee 39</t>
+        </is>
+      </c>
+      <c r="C130" s="3" t="n">
+        <v>46238</v>
+      </c>
+      <c r="D130" s="4" t="n">
+        <v>0.7506944444444444</v>
+      </c>
+      <c r="E130" s="4" t="n">
+        <v>0.4965277777777778</v>
+      </c>
+      <c r="F130" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151849.jpg</t>
+        </is>
+      </c>
+      <c r="G130" s="2" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B131" s="2" t="inlineStr">
+        <is>
+          <t>Employee 39</t>
+        </is>
+      </c>
+      <c r="C131" s="3" t="n">
+        <v>46237</v>
+      </c>
+      <c r="D131" s="4" t="n">
+        <v>0.7472222222222222</v>
+      </c>
+      <c r="E131" s="4" t="n">
+        <v>0.2618055555555556</v>
+      </c>
+      <c r="F131" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151849.jpg</t>
+        </is>
+      </c>
+      <c r="G131" s="2" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>Employee 39</t>
+        </is>
+      </c>
+      <c r="C132" s="3" t="n">
+        <v>46236</v>
+      </c>
+      <c r="D132" s="4" t="n">
+        <v>0.7430555555555556</v>
+      </c>
+      <c r="E132" s="4" t="n">
+        <v>0.2972222222222222</v>
+      </c>
+      <c r="F132" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151849.jpg</t>
+        </is>
+      </c>
+      <c r="G132" s="2" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B133" s="2" t="inlineStr">
+        <is>
+          <t>Employee 39</t>
+        </is>
+      </c>
+      <c r="C133" s="3" t="n">
+        <v>46235</v>
+      </c>
+      <c r="D133" s="4" t="n">
+        <v>0.7319444444444444</v>
+      </c>
+      <c r="E133" s="4" t="n">
+        <v>0.2590277777777778</v>
+      </c>
+      <c r="F133" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151849.jpg</t>
+        </is>
+      </c>
+      <c r="G133" s="2" t="inlineStr">
+        <is>
+          <t>last day of month; final record</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>Employee 40</t>
+        </is>
+      </c>
+      <c r="C134" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="D134" s="2" t="n"/>
+      <c r="E134" s="4" t="n">
+        <v>0.2416666666666667</v>
+      </c>
+      <c r="F134" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151859.jpg</t>
+        </is>
+      </c>
+      <c r="G134" s="2" t="inlineStr">
+        <is>
+          <t>single punch only</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B135" s="2" t="inlineStr">
+        <is>
+          <t>Employee 40</t>
+        </is>
+      </c>
+      <c r="C135" s="3" t="n">
+        <v>46264</v>
+      </c>
+      <c r="D135" s="4" t="n">
+        <v>0.7513888888888889</v>
+      </c>
+      <c r="E135" s="4" t="n">
+        <v>0.2423611111111111</v>
+      </c>
+      <c r="F135" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151859.jpg</t>
+        </is>
+      </c>
+      <c r="G135" s="2" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>Employee 40</t>
+        </is>
+      </c>
+      <c r="C136" s="3" t="n">
+        <v>46263</v>
+      </c>
+      <c r="D136" s="4" t="n">
+        <v>0.7548611111111111</v>
+      </c>
+      <c r="E136" s="4" t="n">
+        <v>0.2444444444444444</v>
+      </c>
+      <c r="F136" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151859.jpg</t>
+        </is>
+      </c>
+      <c r="G136" s="2" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B137" s="2" t="inlineStr">
+        <is>
+          <t>Employee 40</t>
+        </is>
+      </c>
+      <c r="C137" s="3" t="n">
+        <v>46261</v>
+      </c>
+      <c r="D137" s="4" t="n">
+        <v>0.7513888888888889</v>
+      </c>
+      <c r="E137" s="4" t="n">
+        <v>0.2472222222222222</v>
+      </c>
+      <c r="F137" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151859.jpg</t>
+        </is>
+      </c>
+      <c r="G137" s="2" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>Employee 40</t>
+        </is>
+      </c>
+      <c r="C138" s="3" t="n">
+        <v>46260</v>
+      </c>
+      <c r="D138" s="4" t="n">
+        <v>0.7555555555555555</v>
+      </c>
+      <c r="E138" s="4" t="n">
+        <v>0.2465277777777778</v>
+      </c>
+      <c r="F138" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151906.jpg</t>
+        </is>
+      </c>
+      <c r="G138" s="2" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B139" s="2" t="inlineStr">
+        <is>
+          <t>Employee 40</t>
+        </is>
+      </c>
+      <c r="C139" s="3" t="n">
+        <v>46259</v>
+      </c>
+      <c r="D139" s="4" t="n">
+        <v>0.7506944444444444</v>
+      </c>
+      <c r="E139" s="4" t="n">
+        <v>0.2368055555555555</v>
+      </c>
+      <c r="F139" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151906.jpg</t>
+        </is>
+      </c>
+      <c r="G139" s="2" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>Employee 40</t>
+        </is>
+      </c>
+      <c r="C140" s="3" t="n">
+        <v>46258</v>
+      </c>
+      <c r="D140" s="4" t="n">
+        <v>0.7520833333333333</v>
+      </c>
+      <c r="E140" s="4" t="n">
+        <v>0.2347222222222222</v>
+      </c>
+      <c r="F140" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151906.jpg</t>
+        </is>
+      </c>
+      <c r="G140" s="2" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>Employee 40</t>
+        </is>
+      </c>
+      <c r="C141" s="3" t="n">
+        <v>46257</v>
+      </c>
+      <c r="D141" s="4" t="n">
+        <v>0.7527777777777778</v>
+      </c>
+      <c r="E141" s="4" t="n">
+        <v>0.2458333333333333</v>
+      </c>
+      <c r="F141" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151906.jpg</t>
+        </is>
+      </c>
+      <c r="G141" s="2" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>Employee 40</t>
+        </is>
+      </c>
+      <c r="C142" s="3" t="n">
+        <v>46256</v>
+      </c>
+      <c r="D142" s="4" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E142" s="4" t="n">
+        <v>0.2402777777777778</v>
+      </c>
+      <c r="F142" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151910.jpg</t>
+        </is>
+      </c>
+      <c r="G142" s="2" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
+        <is>
+          <t>Employee 40</t>
+        </is>
+      </c>
+      <c r="C143" s="3" t="n">
+        <v>46254</v>
+      </c>
+      <c r="D143" s="4" t="n">
+        <v>0.7520833333333333</v>
+      </c>
+      <c r="E143" s="4" t="n">
+        <v>0.2402777777777778</v>
+      </c>
+      <c r="F143" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151910.jpg</t>
+        </is>
+      </c>
+      <c r="G143" s="2" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>Employee 40</t>
+        </is>
+      </c>
+      <c r="C144" s="3" t="n">
+        <v>46253</v>
+      </c>
+      <c r="D144" s="4" t="n">
+        <v>0.7506944444444444</v>
+      </c>
+      <c r="E144" s="4" t="n">
+        <v>0.2423611111111111</v>
+      </c>
+      <c r="F144" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151910.jpg</t>
+        </is>
+      </c>
+      <c r="G144" s="2" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B145" s="2" t="inlineStr">
+        <is>
+          <t>Employee 40</t>
+        </is>
+      </c>
+      <c r="C145" s="3" t="n">
+        <v>46252</v>
+      </c>
+      <c r="D145" s="4" t="n">
+        <v>0.7527777777777778</v>
+      </c>
+      <c r="E145" s="4" t="n">
+        <v>0.2451388888888889</v>
+      </c>
+      <c r="F145" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151910.jpg</t>
+        </is>
+      </c>
+      <c r="G145" s="2" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>Employee 40</t>
+        </is>
+      </c>
+      <c r="C146" s="3" t="n">
+        <v>46251</v>
+      </c>
+      <c r="D146" s="4" t="n">
+        <v>0.7541666666666667</v>
+      </c>
+      <c r="E146" s="4" t="n">
+        <v>0.2395833333333333</v>
+      </c>
+      <c r="F146" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151915.jpg</t>
+        </is>
+      </c>
+      <c r="G146" s="2" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B147" s="2" t="inlineStr">
+        <is>
+          <t>Employee 40</t>
+        </is>
+      </c>
+      <c r="C147" s="3" t="n">
+        <v>46250</v>
+      </c>
+      <c r="D147" s="4" t="n">
+        <v>0.7520833333333333</v>
+      </c>
+      <c r="E147" s="4" t="n">
+        <v>0.2354166666666667</v>
+      </c>
+      <c r="F147" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151915.jpg</t>
+        </is>
+      </c>
+      <c r="G147" s="2" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>Employee 40</t>
+        </is>
+      </c>
+      <c r="C148" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="D148" s="4" t="n">
+        <v>0.7513888888888889</v>
+      </c>
+      <c r="E148" s="4" t="n">
+        <v>0.2381944444444444</v>
+      </c>
+      <c r="F148" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151915.jpg</t>
+        </is>
+      </c>
+      <c r="G148" s="2" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B149" s="2" t="inlineStr">
+        <is>
+          <t>Employee 40</t>
+        </is>
+      </c>
+      <c r="C149" s="3" t="n">
+        <v>46247</v>
+      </c>
+      <c r="D149" s="4" t="n">
+        <v>0.7576388888888889</v>
+      </c>
+      <c r="E149" s="4" t="n">
+        <v>0.2444444444444444</v>
+      </c>
+      <c r="F149" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151915.jpg</t>
+        </is>
+      </c>
+      <c r="G149" s="2" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
+          <t>Employee 40</t>
+        </is>
+      </c>
+      <c r="C150" s="3" t="n">
+        <v>46246</v>
+      </c>
+      <c r="D150" s="2" t="n"/>
+      <c r="E150" s="2" t="n"/>
+      <c r="F150" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151915.jpg</t>
+        </is>
+      </c>
+      <c r="G150" s="2" t="inlineStr">
+        <is>
+          <t>PLEASE VERIFY: check-in/out times not captured (gap between source photos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B151" s="2" t="inlineStr">
+        <is>
+          <t>Employee 40</t>
+        </is>
+      </c>
+      <c r="C151" s="3" t="n">
+        <v>46242</v>
+      </c>
+      <c r="D151" s="4" t="n">
+        <v>0.7548611111111111</v>
+      </c>
+      <c r="E151" s="4" t="n">
+        <v>0.2430555555555556</v>
+      </c>
+      <c r="F151" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151924.jpg</t>
+        </is>
+      </c>
+      <c r="G151" s="2" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>Employee 40</t>
+        </is>
+      </c>
+      <c r="C152" s="3" t="n">
+        <v>46240</v>
+      </c>
+      <c r="D152" s="4" t="n">
+        <v>0.7513888888888889</v>
+      </c>
+      <c r="E152" s="4" t="n">
+        <v>0.2402777777777778</v>
+      </c>
+      <c r="F152" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151924.jpg</t>
+        </is>
+      </c>
+      <c r="G152" s="2" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B153" s="2" t="inlineStr">
+        <is>
+          <t>Employee 40</t>
+        </is>
+      </c>
+      <c r="C153" s="3" t="n">
+        <v>46239</v>
+      </c>
+      <c r="D153" s="4" t="n">
+        <v>0.7611111111111111</v>
+      </c>
+      <c r="E153" s="4" t="n">
+        <v>0.2368055555555555</v>
+      </c>
+      <c r="F153" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151924.jpg</t>
+        </is>
+      </c>
+      <c r="G153" s="2" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>Employee 40</t>
+        </is>
+      </c>
+      <c r="C154" s="3" t="n">
+        <v>46238</v>
+      </c>
+      <c r="D154" s="4" t="n">
+        <v>0.7520833333333333</v>
+      </c>
+      <c r="E154" s="4" t="n">
+        <v>0.2451388888888889</v>
+      </c>
+      <c r="F154" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151924.jpg</t>
+        </is>
+      </c>
+      <c r="G154" s="2" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B155" s="2" t="inlineStr">
+        <is>
+          <t>Employee 40</t>
+        </is>
+      </c>
+      <c r="C155" s="3" t="n">
+        <v>46237</v>
+      </c>
+      <c r="D155" s="4" t="n">
+        <v>0.7527777777777778</v>
+      </c>
+      <c r="E155" s="4" t="n">
+        <v>0.24375</v>
+      </c>
+      <c r="F155" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151928.jpg</t>
+        </is>
+      </c>
+      <c r="G155" s="2" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>Employee 40</t>
+        </is>
+      </c>
+      <c r="C156" s="3" t="n">
+        <v>46236</v>
+      </c>
+      <c r="D156" s="4" t="n">
+        <v>0.7520833333333333</v>
+      </c>
+      <c r="E156" s="4" t="n">
+        <v>0.24375</v>
+      </c>
+      <c r="F156" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151928.jpg</t>
+        </is>
+      </c>
+      <c r="G156" s="2" t="inlineStr"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B157" s="2" t="inlineStr">
+        <is>
+          <t>Employee 40</t>
+        </is>
+      </c>
+      <c r="C157" s="3" t="n">
+        <v>46235</v>
+      </c>
+      <c r="D157" s="4" t="n">
+        <v>0.7506944444444444</v>
+      </c>
+      <c r="E157" s="4" t="n">
+        <v>0.2451388888888889</v>
+      </c>
+      <c r="F157" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151928.jpg</t>
+        </is>
+      </c>
+      <c r="G157" s="2" t="inlineStr">
+        <is>
+          <t>last day of month; final record</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Extract punch data for employees 41, 42, 44 (folder 2 batch)
Covers 60 of ~80 uploaded images now (folders 2, 3, 4 complete).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PeUzxoX8Admt6BxLMC3Cdz
</commit_message>
<xml_diff>
--- a/output/timesheet.xlsx
+++ b/output/timesheet.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G157"/>
+  <dimension ref="A1:G234"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4775,6 +4775,2157 @@
         </is>
       </c>
     </row>
+    <row r="158">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B158" s="2" t="inlineStr">
+        <is>
+          <t>Employee 41</t>
+        </is>
+      </c>
+      <c r="C158" s="3" t="n">
+        <v>46264</v>
+      </c>
+      <c r="D158" s="4" t="n">
+        <v>0.7215277777777778</v>
+      </c>
+      <c r="E158" s="4" t="n">
+        <v>0.2958333333333333</v>
+      </c>
+      <c r="F158" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151937.jpg</t>
+        </is>
+      </c>
+      <c r="G158" s="2" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B159" s="2" t="inlineStr">
+        <is>
+          <t>Employee 41</t>
+        </is>
+      </c>
+      <c r="C159" s="3" t="n">
+        <v>46263</v>
+      </c>
+      <c r="D159" s="4" t="n">
+        <v>0.7104166666666667</v>
+      </c>
+      <c r="E159" s="4" t="n">
+        <v>0.2513888888888889</v>
+      </c>
+      <c r="F159" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151937.jpg</t>
+        </is>
+      </c>
+      <c r="G159" s="2" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B160" s="2" t="inlineStr">
+        <is>
+          <t>Employee 41</t>
+        </is>
+      </c>
+      <c r="C160" s="3" t="n">
+        <v>46261</v>
+      </c>
+      <c r="D160" s="4" t="n">
+        <v>0.7111111111111111</v>
+      </c>
+      <c r="E160" s="4" t="n">
+        <v>0.4881944444444444</v>
+      </c>
+      <c r="F160" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151937.jpg</t>
+        </is>
+      </c>
+      <c r="G160" s="2" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B161" s="2" t="inlineStr">
+        <is>
+          <t>Employee 41</t>
+        </is>
+      </c>
+      <c r="C161" s="3" t="n">
+        <v>46260</v>
+      </c>
+      <c r="D161" s="4" t="n">
+        <v>0.7152777777777778</v>
+      </c>
+      <c r="E161" s="4" t="n">
+        <v>0.2375</v>
+      </c>
+      <c r="F161" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151937.jpg</t>
+        </is>
+      </c>
+      <c r="G161" s="2" t="inlineStr"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B162" s="2" t="inlineStr">
+        <is>
+          <t>Employee 41</t>
+        </is>
+      </c>
+      <c r="C162" s="3" t="n">
+        <v>46259</v>
+      </c>
+      <c r="D162" s="4" t="n">
+        <v>0.7222222222222222</v>
+      </c>
+      <c r="E162" s="4" t="n">
+        <v>0.2854166666666667</v>
+      </c>
+      <c r="F162" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151944.jpg</t>
+        </is>
+      </c>
+      <c r="G162" s="2" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B163" s="2" t="inlineStr">
+        <is>
+          <t>Employee 41</t>
+        </is>
+      </c>
+      <c r="C163" s="3" t="n">
+        <v>46258</v>
+      </c>
+      <c r="D163" s="4" t="n">
+        <v>0.7055555555555556</v>
+      </c>
+      <c r="E163" s="4" t="n">
+        <v>0.2784722222222222</v>
+      </c>
+      <c r="F163" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151944.jpg</t>
+        </is>
+      </c>
+      <c r="G163" s="2" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B164" s="2" t="inlineStr">
+        <is>
+          <t>Employee 41</t>
+        </is>
+      </c>
+      <c r="C164" s="3" t="n">
+        <v>46257</v>
+      </c>
+      <c r="D164" s="4" t="n">
+        <v>0.7076388888888889</v>
+      </c>
+      <c r="E164" s="4" t="n">
+        <v>0.2444444444444444</v>
+      </c>
+      <c r="F164" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151944.jpg</t>
+        </is>
+      </c>
+      <c r="G164" s="2" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B165" s="2" t="inlineStr">
+        <is>
+          <t>Employee 41</t>
+        </is>
+      </c>
+      <c r="C165" s="3" t="n">
+        <v>46256</v>
+      </c>
+      <c r="D165" s="4" t="n">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="E165" s="4" t="n">
+        <v>0.2888888888888889</v>
+      </c>
+      <c r="F165" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151944.jpg</t>
+        </is>
+      </c>
+      <c r="G165" s="2" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B166" s="2" t="inlineStr">
+        <is>
+          <t>Employee 41</t>
+        </is>
+      </c>
+      <c r="C166" s="3" t="n">
+        <v>46254</v>
+      </c>
+      <c r="D166" s="4" t="n">
+        <v>0.70625</v>
+      </c>
+      <c r="E166" s="4" t="n">
+        <v>0.4298611111111111</v>
+      </c>
+      <c r="F166" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151952.jpg</t>
+        </is>
+      </c>
+      <c r="G166" s="2" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B167" s="2" t="inlineStr">
+        <is>
+          <t>Employee 41</t>
+        </is>
+      </c>
+      <c r="C167" s="3" t="n">
+        <v>46253</v>
+      </c>
+      <c r="D167" s="4" t="n">
+        <v>0.7305555555555555</v>
+      </c>
+      <c r="E167" s="4" t="n">
+        <v>0.2944444444444445</v>
+      </c>
+      <c r="F167" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151952.jpg</t>
+        </is>
+      </c>
+      <c r="G167" s="2" t="inlineStr"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B168" s="2" t="inlineStr">
+        <is>
+          <t>Employee 41</t>
+        </is>
+      </c>
+      <c r="C168" s="3" t="n">
+        <v>46252</v>
+      </c>
+      <c r="D168" s="4" t="n">
+        <v>0.7208333333333333</v>
+      </c>
+      <c r="E168" s="4" t="n">
+        <v>0.3659722222222222</v>
+      </c>
+      <c r="F168" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151952.jpg</t>
+        </is>
+      </c>
+      <c r="G168" s="2" t="inlineStr"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B169" s="2" t="inlineStr">
+        <is>
+          <t>Employee 41</t>
+        </is>
+      </c>
+      <c r="C169" s="3" t="n">
+        <v>46251</v>
+      </c>
+      <c r="D169" s="4" t="n">
+        <v>0.7069444444444445</v>
+      </c>
+      <c r="E169" s="4" t="n">
+        <v>0.3104166666666667</v>
+      </c>
+      <c r="F169" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_151952.jpg</t>
+        </is>
+      </c>
+      <c r="G169" s="2" t="inlineStr"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B170" s="2" t="inlineStr">
+        <is>
+          <t>Employee 41</t>
+        </is>
+      </c>
+      <c r="C170" s="3" t="n">
+        <v>46250</v>
+      </c>
+      <c r="D170" s="4" t="n">
+        <v>0.7173611111111111</v>
+      </c>
+      <c r="E170" s="4" t="n">
+        <v>0.3416666666666667</v>
+      </c>
+      <c r="F170" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152000.jpg</t>
+        </is>
+      </c>
+      <c r="G170" s="2" t="inlineStr"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B171" s="2" t="inlineStr">
+        <is>
+          <t>Employee 41</t>
+        </is>
+      </c>
+      <c r="C171" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="D171" s="4" t="n">
+        <v>0.7625</v>
+      </c>
+      <c r="E171" s="4" t="n">
+        <v>0.2680555555555555</v>
+      </c>
+      <c r="F171" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152000.jpg</t>
+        </is>
+      </c>
+      <c r="G171" s="2" t="inlineStr"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B172" s="2" t="inlineStr">
+        <is>
+          <t>Employee 41</t>
+        </is>
+      </c>
+      <c r="C172" s="3" t="n">
+        <v>46247</v>
+      </c>
+      <c r="D172" s="4" t="n">
+        <v>0.7583333333333333</v>
+      </c>
+      <c r="E172" s="4" t="n">
+        <v>0.3409722222222222</v>
+      </c>
+      <c r="F172" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152000.jpg</t>
+        </is>
+      </c>
+      <c r="G172" s="2" t="inlineStr"/>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B173" s="2" t="inlineStr">
+        <is>
+          <t>Employee 41</t>
+        </is>
+      </c>
+      <c r="C173" s="3" t="n">
+        <v>46246</v>
+      </c>
+      <c r="D173" s="4" t="n">
+        <v>0.7222222222222222</v>
+      </c>
+      <c r="E173" s="4" t="n">
+        <v>0.2694444444444444</v>
+      </c>
+      <c r="F173" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152000.jpg</t>
+        </is>
+      </c>
+      <c r="G173" s="2" t="inlineStr"/>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B174" s="2" t="inlineStr">
+        <is>
+          <t>Employee 41</t>
+        </is>
+      </c>
+      <c r="C174" s="3" t="n">
+        <v>46245</v>
+      </c>
+      <c r="D174" s="4" t="n">
+        <v>0.7618055555555555</v>
+      </c>
+      <c r="E174" s="4" t="n">
+        <v>0.275</v>
+      </c>
+      <c r="F174" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152000.jpg</t>
+        </is>
+      </c>
+      <c r="G174" s="2" t="inlineStr"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B175" s="2" t="inlineStr">
+        <is>
+          <t>Employee 41</t>
+        </is>
+      </c>
+      <c r="C175" s="3" t="n">
+        <v>46244</v>
+      </c>
+      <c r="D175" s="4" t="n">
+        <v>0.75625</v>
+      </c>
+      <c r="E175" s="4" t="n">
+        <v>0.2298611111111111</v>
+      </c>
+      <c r="F175" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152006.jpg</t>
+        </is>
+      </c>
+      <c r="G175" s="2" t="inlineStr">
+        <is>
+          <t>extra punch: 06:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B176" s="2" t="inlineStr">
+        <is>
+          <t>Employee 41</t>
+        </is>
+      </c>
+      <c r="C176" s="3" t="n">
+        <v>46243</v>
+      </c>
+      <c r="D176" s="4" t="n">
+        <v>0.7694444444444445</v>
+      </c>
+      <c r="E176" s="4" t="n">
+        <v>0.2451388888888889</v>
+      </c>
+      <c r="F176" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152006.jpg</t>
+        </is>
+      </c>
+      <c r="G176" s="2" t="inlineStr"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B177" s="2" t="inlineStr">
+        <is>
+          <t>Employee 41</t>
+        </is>
+      </c>
+      <c r="C177" s="3" t="n">
+        <v>46242</v>
+      </c>
+      <c r="D177" s="4" t="n">
+        <v>0.6965277777777777</v>
+      </c>
+      <c r="E177" s="4" t="n">
+        <v>0.2388888888888889</v>
+      </c>
+      <c r="F177" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152006.jpg</t>
+        </is>
+      </c>
+      <c r="G177" s="2" t="inlineStr"/>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B178" s="2" t="inlineStr">
+        <is>
+          <t>Employee 41</t>
+        </is>
+      </c>
+      <c r="C178" s="3" t="n">
+        <v>46240</v>
+      </c>
+      <c r="D178" s="2" t="n"/>
+      <c r="E178" s="4" t="n">
+        <v>0.2715277777777778</v>
+      </c>
+      <c r="F178" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152012.jpg</t>
+        </is>
+      </c>
+      <c r="G178" s="2" t="inlineStr">
+        <is>
+          <t>single punch only</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="2" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B179" s="2" t="inlineStr">
+        <is>
+          <t>Employee 41</t>
+        </is>
+      </c>
+      <c r="C179" s="3" t="n">
+        <v>46239</v>
+      </c>
+      <c r="D179" s="4" t="n">
+        <v>0.7152777777777778</v>
+      </c>
+      <c r="E179" s="4" t="n">
+        <v>0.2756944444444445</v>
+      </c>
+      <c r="F179" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152012.jpg</t>
+        </is>
+      </c>
+      <c r="G179" s="2" t="inlineStr"/>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B180" s="2" t="inlineStr">
+        <is>
+          <t>Employee 41</t>
+        </is>
+      </c>
+      <c r="C180" s="3" t="n">
+        <v>46238</v>
+      </c>
+      <c r="D180" s="4" t="n">
+        <v>0.7527777777777778</v>
+      </c>
+      <c r="E180" s="4" t="n">
+        <v>0.2729166666666666</v>
+      </c>
+      <c r="F180" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152012.jpg</t>
+        </is>
+      </c>
+      <c r="G180" s="2" t="inlineStr"/>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B181" s="2" t="inlineStr">
+        <is>
+          <t>Employee 41</t>
+        </is>
+      </c>
+      <c r="C181" s="3" t="n">
+        <v>46237</v>
+      </c>
+      <c r="D181" s="4" t="n">
+        <v>0.7201388888888889</v>
+      </c>
+      <c r="E181" s="4" t="n">
+        <v>0.2451388888888889</v>
+      </c>
+      <c r="F181" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152012.jpg</t>
+        </is>
+      </c>
+      <c r="G181" s="2" t="inlineStr"/>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B182" s="2" t="inlineStr">
+        <is>
+          <t>Employee 41</t>
+        </is>
+      </c>
+      <c r="C182" s="3" t="n">
+        <v>46236</v>
+      </c>
+      <c r="D182" s="4" t="n">
+        <v>0.7722222222222223</v>
+      </c>
+      <c r="E182" s="4" t="n">
+        <v>0.2722222222222222</v>
+      </c>
+      <c r="F182" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152017.jpg</t>
+        </is>
+      </c>
+      <c r="G182" s="2" t="inlineStr"/>
+    </row>
+    <row r="183">
+      <c r="A183" s="2" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B183" s="2" t="inlineStr">
+        <is>
+          <t>Employee 41</t>
+        </is>
+      </c>
+      <c r="C183" s="3" t="n">
+        <v>46235</v>
+      </c>
+      <c r="D183" s="4" t="n">
+        <v>0.7854166666666667</v>
+      </c>
+      <c r="E183" s="4" t="n">
+        <v>0.275</v>
+      </c>
+      <c r="F183" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152017.jpg</t>
+        </is>
+      </c>
+      <c r="G183" s="2" t="inlineStr">
+        <is>
+          <t>last day of month; final record</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B184" s="2" t="inlineStr">
+        <is>
+          <t>Employee 42</t>
+        </is>
+      </c>
+      <c r="C184" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="D184" s="2" t="n"/>
+      <c r="E184" s="4" t="n">
+        <v>0.3888888888888889</v>
+      </c>
+      <c r="F184" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152028.jpg</t>
+        </is>
+      </c>
+      <c r="G184" s="2" t="inlineStr">
+        <is>
+          <t>single punch only</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B185" s="2" t="inlineStr">
+        <is>
+          <t>Employee 42</t>
+        </is>
+      </c>
+      <c r="C185" s="3" t="n">
+        <v>46264</v>
+      </c>
+      <c r="D185" s="4" t="n">
+        <v>0.7472222222222222</v>
+      </c>
+      <c r="E185" s="4" t="n">
+        <v>0.2798611111111111</v>
+      </c>
+      <c r="F185" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152028.jpg</t>
+        </is>
+      </c>
+      <c r="G185" s="2" t="inlineStr"/>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B186" s="2" t="inlineStr">
+        <is>
+          <t>Employee 42</t>
+        </is>
+      </c>
+      <c r="C186" s="3" t="n">
+        <v>46263</v>
+      </c>
+      <c r="D186" s="4" t="n">
+        <v>0.7291666666666666</v>
+      </c>
+      <c r="E186" s="2" t="n"/>
+      <c r="F186" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152028.jpg</t>
+        </is>
+      </c>
+      <c r="G186" s="2" t="inlineStr">
+        <is>
+          <t>single punch only</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B187" s="2" t="inlineStr">
+        <is>
+          <t>Employee 42</t>
+        </is>
+      </c>
+      <c r="C187" s="3" t="n">
+        <v>46261</v>
+      </c>
+      <c r="D187" s="4" t="n">
+        <v>0.8645833333333334</v>
+      </c>
+      <c r="E187" s="4" t="n">
+        <v>0.2833333333333333</v>
+      </c>
+      <c r="F187" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152028.jpg</t>
+        </is>
+      </c>
+      <c r="G187" s="2" t="inlineStr"/>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B188" s="2" t="inlineStr">
+        <is>
+          <t>Employee 42</t>
+        </is>
+      </c>
+      <c r="C188" s="3" t="n">
+        <v>46260</v>
+      </c>
+      <c r="D188" s="4" t="n">
+        <v>0.6986111111111111</v>
+      </c>
+      <c r="E188" s="2" t="n"/>
+      <c r="F188" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152039.jpg</t>
+        </is>
+      </c>
+      <c r="G188" s="2" t="inlineStr">
+        <is>
+          <t>single punch only</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B189" s="2" t="inlineStr">
+        <is>
+          <t>Employee 42</t>
+        </is>
+      </c>
+      <c r="C189" s="3" t="n">
+        <v>46259</v>
+      </c>
+      <c r="D189" s="4" t="n">
+        <v>0.6895833333333333</v>
+      </c>
+      <c r="E189" s="4" t="n">
+        <v>0.2868055555555555</v>
+      </c>
+      <c r="F189" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152039.jpg</t>
+        </is>
+      </c>
+      <c r="G189" s="2" t="inlineStr"/>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B190" s="2" t="inlineStr">
+        <is>
+          <t>Employee 42</t>
+        </is>
+      </c>
+      <c r="C190" s="3" t="n">
+        <v>46258</v>
+      </c>
+      <c r="D190" s="4" t="n">
+        <v>0.7506944444444444</v>
+      </c>
+      <c r="E190" s="2" t="n"/>
+      <c r="F190" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152039.jpg</t>
+        </is>
+      </c>
+      <c r="G190" s="2" t="inlineStr">
+        <is>
+          <t>single punch only</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B191" s="2" t="inlineStr">
+        <is>
+          <t>Employee 42</t>
+        </is>
+      </c>
+      <c r="C191" s="3" t="n">
+        <v>46257</v>
+      </c>
+      <c r="D191" s="4" t="n">
+        <v>0.7569444444444444</v>
+      </c>
+      <c r="E191" s="4" t="n">
+        <v>0.2548611111111111</v>
+      </c>
+      <c r="F191" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152039.jpg</t>
+        </is>
+      </c>
+      <c r="G191" s="2" t="inlineStr"/>
+    </row>
+    <row r="192">
+      <c r="A192" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B192" s="2" t="inlineStr">
+        <is>
+          <t>Employee 42</t>
+        </is>
+      </c>
+      <c r="C192" s="3" t="n">
+        <v>46256</v>
+      </c>
+      <c r="D192" s="4" t="n">
+        <v>0.74375</v>
+      </c>
+      <c r="E192" s="2" t="n"/>
+      <c r="F192" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152049.jpg</t>
+        </is>
+      </c>
+      <c r="G192" s="2" t="inlineStr">
+        <is>
+          <t>single punch only</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B193" s="2" t="inlineStr">
+        <is>
+          <t>Employee 42</t>
+        </is>
+      </c>
+      <c r="C193" s="3" t="n">
+        <v>46254</v>
+      </c>
+      <c r="D193" s="2" t="n"/>
+      <c r="E193" s="4" t="n">
+        <v>0.2868055555555555</v>
+      </c>
+      <c r="F193" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152049.jpg</t>
+        </is>
+      </c>
+      <c r="G193" s="2" t="inlineStr">
+        <is>
+          <t>single punch only</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B194" s="2" t="inlineStr">
+        <is>
+          <t>Employee 42</t>
+        </is>
+      </c>
+      <c r="C194" s="3" t="n">
+        <v>46253</v>
+      </c>
+      <c r="D194" s="4" t="n">
+        <v>0.74375</v>
+      </c>
+      <c r="E194" s="4" t="n">
+        <v>0.3166666666666667</v>
+      </c>
+      <c r="F194" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152049.jpg</t>
+        </is>
+      </c>
+      <c r="G194" s="2" t="inlineStr">
+        <is>
+          <t>extra punch: 08:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B195" s="2" t="inlineStr">
+        <is>
+          <t>Employee 42</t>
+        </is>
+      </c>
+      <c r="C195" s="3" t="n">
+        <v>46252</v>
+      </c>
+      <c r="D195" s="4" t="n">
+        <v>0.7645833333333333</v>
+      </c>
+      <c r="E195" s="4" t="n">
+        <v>0.28125</v>
+      </c>
+      <c r="F195" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152049.jpg</t>
+        </is>
+      </c>
+      <c r="G195" s="2" t="inlineStr"/>
+    </row>
+    <row r="196">
+      <c r="A196" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B196" s="2" t="inlineStr">
+        <is>
+          <t>Employee 42</t>
+        </is>
+      </c>
+      <c r="C196" s="3" t="n">
+        <v>46251</v>
+      </c>
+      <c r="D196" s="4" t="n">
+        <v>0.7326388888888888</v>
+      </c>
+      <c r="E196" s="4" t="n">
+        <v>0.2833333333333333</v>
+      </c>
+      <c r="F196" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152053.jpg</t>
+        </is>
+      </c>
+      <c r="G196" s="2" t="inlineStr"/>
+    </row>
+    <row r="197">
+      <c r="A197" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B197" s="2" t="inlineStr">
+        <is>
+          <t>Employee 42</t>
+        </is>
+      </c>
+      <c r="C197" s="3" t="n">
+        <v>46250</v>
+      </c>
+      <c r="D197" s="4" t="n">
+        <v>0.7104166666666667</v>
+      </c>
+      <c r="E197" s="4" t="n">
+        <v>0.3409722222222222</v>
+      </c>
+      <c r="F197" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152053.jpg</t>
+        </is>
+      </c>
+      <c r="G197" s="2" t="inlineStr"/>
+    </row>
+    <row r="198">
+      <c r="A198" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B198" s="2" t="inlineStr">
+        <is>
+          <t>Employee 42</t>
+        </is>
+      </c>
+      <c r="C198" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="D198" s="4" t="n">
+        <v>0.7270833333333333</v>
+      </c>
+      <c r="E198" s="4" t="n">
+        <v>0.2423611111111111</v>
+      </c>
+      <c r="F198" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152053.jpg</t>
+        </is>
+      </c>
+      <c r="G198" s="2" t="inlineStr">
+        <is>
+          <t>extra punches: 17:27 07:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B199" s="2" t="inlineStr">
+        <is>
+          <t>Employee 42</t>
+        </is>
+      </c>
+      <c r="C199" s="3" t="n">
+        <v>46247</v>
+      </c>
+      <c r="D199" s="4" t="n">
+        <v>0.7236111111111111</v>
+      </c>
+      <c r="E199" s="4" t="n">
+        <v>0.3388888888888889</v>
+      </c>
+      <c r="F199" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152053.jpg</t>
+        </is>
+      </c>
+      <c r="G199" s="2" t="inlineStr">
+        <is>
+          <t>extra punch: 17:21</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B200" s="2" t="inlineStr">
+        <is>
+          <t>Employee 42</t>
+        </is>
+      </c>
+      <c r="C200" s="3" t="n">
+        <v>46246</v>
+      </c>
+      <c r="D200" s="4" t="n">
+        <v>0.7222222222222222</v>
+      </c>
+      <c r="E200" s="4" t="n">
+        <v>0.2548611111111111</v>
+      </c>
+      <c r="F200" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152058.jpg</t>
+        </is>
+      </c>
+      <c r="G200" s="2" t="inlineStr">
+        <is>
+          <t>extra punches: 07:44 06:16</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B201" s="2" t="inlineStr">
+        <is>
+          <t>Employee 42</t>
+        </is>
+      </c>
+      <c r="C201" s="3" t="n">
+        <v>46245</v>
+      </c>
+      <c r="D201" s="4" t="n">
+        <v>0.7465277777777778</v>
+      </c>
+      <c r="E201" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F201" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152058.jpg</t>
+        </is>
+      </c>
+      <c r="G201" s="2" t="inlineStr"/>
+    </row>
+    <row r="202">
+      <c r="A202" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B202" s="2" t="inlineStr">
+        <is>
+          <t>Employee 42</t>
+        </is>
+      </c>
+      <c r="C202" s="3" t="n">
+        <v>46244</v>
+      </c>
+      <c r="D202" s="4" t="n">
+        <v>0.7479166666666667</v>
+      </c>
+      <c r="E202" s="4" t="n">
+        <v>0.2875</v>
+      </c>
+      <c r="F202" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152058.jpg</t>
+        </is>
+      </c>
+      <c r="G202" s="2" t="inlineStr"/>
+    </row>
+    <row r="203">
+      <c r="A203" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B203" s="2" t="inlineStr">
+        <is>
+          <t>Employee 42</t>
+        </is>
+      </c>
+      <c r="C203" s="3" t="n">
+        <v>46243</v>
+      </c>
+      <c r="D203" s="4" t="n">
+        <v>0.7555555555555555</v>
+      </c>
+      <c r="E203" s="4" t="n">
+        <v>0.2784722222222222</v>
+      </c>
+      <c r="F203" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152058.jpg</t>
+        </is>
+      </c>
+      <c r="G203" s="2" t="inlineStr"/>
+    </row>
+    <row r="204">
+      <c r="A204" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B204" s="2" t="inlineStr">
+        <is>
+          <t>Employee 42</t>
+        </is>
+      </c>
+      <c r="C204" s="3" t="n">
+        <v>46242</v>
+      </c>
+      <c r="D204" s="4" t="n">
+        <v>0.7284722222222222</v>
+      </c>
+      <c r="E204" s="4" t="n">
+        <v>0.2791666666666667</v>
+      </c>
+      <c r="F204" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152106.jpg</t>
+        </is>
+      </c>
+      <c r="G204" s="2" t="inlineStr"/>
+    </row>
+    <row r="205">
+      <c r="A205" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B205" s="2" t="inlineStr">
+        <is>
+          <t>Employee 42</t>
+        </is>
+      </c>
+      <c r="C205" s="3" t="n">
+        <v>46240</v>
+      </c>
+      <c r="D205" s="4" t="n">
+        <v>0.7277777777777777</v>
+      </c>
+      <c r="E205" s="4" t="n">
+        <v>0.3986111111111111</v>
+      </c>
+      <c r="F205" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152106.jpg</t>
+        </is>
+      </c>
+      <c r="G205" s="2" t="inlineStr"/>
+    </row>
+    <row r="206">
+      <c r="A206" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B206" s="2" t="inlineStr">
+        <is>
+          <t>Employee 42</t>
+        </is>
+      </c>
+      <c r="C206" s="3" t="n">
+        <v>46239</v>
+      </c>
+      <c r="D206" s="4" t="n">
+        <v>0.7715277777777778</v>
+      </c>
+      <c r="E206" s="2" t="n"/>
+      <c r="F206" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152106.jpg</t>
+        </is>
+      </c>
+      <c r="G206" s="2" t="inlineStr">
+        <is>
+          <t>single punch only</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B207" s="2" t="inlineStr">
+        <is>
+          <t>Employee 42</t>
+        </is>
+      </c>
+      <c r="C207" s="3" t="n">
+        <v>46238</v>
+      </c>
+      <c r="D207" s="4" t="n">
+        <v>0.7263888888888889</v>
+      </c>
+      <c r="E207" s="4" t="n">
+        <v>0.3305555555555555</v>
+      </c>
+      <c r="F207" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152106.jpg</t>
+        </is>
+      </c>
+      <c r="G207" s="2" t="inlineStr"/>
+    </row>
+    <row r="208">
+      <c r="A208" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B208" s="2" t="inlineStr">
+        <is>
+          <t>Employee 42</t>
+        </is>
+      </c>
+      <c r="C208" s="3" t="n">
+        <v>46237</v>
+      </c>
+      <c r="D208" s="4" t="n">
+        <v>0.7111111111111111</v>
+      </c>
+      <c r="E208" s="4" t="n">
+        <v>0.3291666666666667</v>
+      </c>
+      <c r="F208" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152113.jpg</t>
+        </is>
+      </c>
+      <c r="G208" s="2" t="inlineStr"/>
+    </row>
+    <row r="209">
+      <c r="A209" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B209" s="2" t="inlineStr">
+        <is>
+          <t>Employee 42</t>
+        </is>
+      </c>
+      <c r="C209" s="3" t="n">
+        <v>46236</v>
+      </c>
+      <c r="D209" s="4" t="n">
+        <v>0.3583333333333333</v>
+      </c>
+      <c r="E209" s="2" t="n"/>
+      <c r="F209" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152113.jpg</t>
+        </is>
+      </c>
+      <c r="G209" s="2" t="inlineStr">
+        <is>
+          <t>single punch only</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B210" s="2" t="inlineStr">
+        <is>
+          <t>Employee 42</t>
+        </is>
+      </c>
+      <c r="C210" s="3" t="n">
+        <v>46235</v>
+      </c>
+      <c r="D210" s="4" t="n">
+        <v>0.7347222222222223</v>
+      </c>
+      <c r="E210" s="4" t="n">
+        <v>0.3305555555555555</v>
+      </c>
+      <c r="F210" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152113.jpg</t>
+        </is>
+      </c>
+      <c r="G210" s="2" t="inlineStr">
+        <is>
+          <t>last day of month; final record</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B211" s="2" t="inlineStr">
+        <is>
+          <t>Employee 44</t>
+        </is>
+      </c>
+      <c r="C211" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="D211" s="2" t="n"/>
+      <c r="E211" s="4" t="n">
+        <v>0.2569444444444444</v>
+      </c>
+      <c r="F211" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152124.jpg</t>
+        </is>
+      </c>
+      <c r="G211" s="2" t="inlineStr">
+        <is>
+          <t>single punch only</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B212" s="2" t="inlineStr">
+        <is>
+          <t>Employee 44</t>
+        </is>
+      </c>
+      <c r="C212" s="3" t="n">
+        <v>46264</v>
+      </c>
+      <c r="D212" s="4" t="n">
+        <v>0.7458333333333333</v>
+      </c>
+      <c r="E212" s="4" t="n">
+        <v>0.2555555555555555</v>
+      </c>
+      <c r="F212" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152124.jpg</t>
+        </is>
+      </c>
+      <c r="G212" s="2" t="inlineStr"/>
+    </row>
+    <row r="213">
+      <c r="A213" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B213" s="2" t="inlineStr">
+        <is>
+          <t>Employee 44</t>
+        </is>
+      </c>
+      <c r="C213" s="3" t="n">
+        <v>46263</v>
+      </c>
+      <c r="D213" s="4" t="n">
+        <v>0.7444444444444445</v>
+      </c>
+      <c r="E213" s="4" t="n">
+        <v>0.2201388888888889</v>
+      </c>
+      <c r="F213" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152124.jpg</t>
+        </is>
+      </c>
+      <c r="G213" s="2" t="inlineStr"/>
+    </row>
+    <row r="214">
+      <c r="A214" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B214" s="2" t="inlineStr">
+        <is>
+          <t>Employee 44</t>
+        </is>
+      </c>
+      <c r="C214" s="3" t="n">
+        <v>46261</v>
+      </c>
+      <c r="D214" s="4" t="n">
+        <v>0.7569444444444444</v>
+      </c>
+      <c r="E214" s="4" t="n">
+        <v>0.2722222222222222</v>
+      </c>
+      <c r="F214" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152124.jpg</t>
+        </is>
+      </c>
+      <c r="G214" s="2" t="inlineStr"/>
+    </row>
+    <row r="215">
+      <c r="A215" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B215" s="2" t="inlineStr">
+        <is>
+          <t>Employee 44</t>
+        </is>
+      </c>
+      <c r="C215" s="3" t="n">
+        <v>46260</v>
+      </c>
+      <c r="D215" s="4" t="n">
+        <v>0.7541666666666667</v>
+      </c>
+      <c r="E215" s="4" t="n">
+        <v>0.2555555555555555</v>
+      </c>
+      <c r="F215" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152137.jpg</t>
+        </is>
+      </c>
+      <c r="G215" s="2" t="inlineStr"/>
+    </row>
+    <row r="216">
+      <c r="A216" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B216" s="2" t="inlineStr">
+        <is>
+          <t>Employee 44</t>
+        </is>
+      </c>
+      <c r="C216" s="3" t="n">
+        <v>46259</v>
+      </c>
+      <c r="D216" s="4" t="n">
+        <v>0.7541666666666667</v>
+      </c>
+      <c r="E216" s="4" t="n">
+        <v>0.3555555555555556</v>
+      </c>
+      <c r="F216" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152137.jpg</t>
+        </is>
+      </c>
+      <c r="G216" s="2" t="inlineStr">
+        <is>
+          <t>extra punch: 06:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B217" s="2" t="inlineStr">
+        <is>
+          <t>Employee 44</t>
+        </is>
+      </c>
+      <c r="C217" s="3" t="n">
+        <v>46258</v>
+      </c>
+      <c r="D217" s="4" t="n">
+        <v>0.7513888888888889</v>
+      </c>
+      <c r="E217" s="4" t="n">
+        <v>0.2319444444444445</v>
+      </c>
+      <c r="F217" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152137.jpg</t>
+        </is>
+      </c>
+      <c r="G217" s="2" t="inlineStr">
+        <is>
+          <t>extra punch: 18:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B218" s="2" t="inlineStr">
+        <is>
+          <t>Employee 44</t>
+        </is>
+      </c>
+      <c r="C218" s="3" t="n">
+        <v>46257</v>
+      </c>
+      <c r="D218" s="4" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E218" s="4" t="n">
+        <v>0.2402777777777778</v>
+      </c>
+      <c r="F218" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152137.jpg</t>
+        </is>
+      </c>
+      <c r="G218" s="2" t="inlineStr"/>
+    </row>
+    <row r="219">
+      <c r="A219" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B219" s="2" t="inlineStr">
+        <is>
+          <t>Employee 44</t>
+        </is>
+      </c>
+      <c r="C219" s="3" t="n">
+        <v>46256</v>
+      </c>
+      <c r="D219" s="4" t="n">
+        <v>0.74375</v>
+      </c>
+      <c r="E219" s="4" t="n">
+        <v>0.2402777777777778</v>
+      </c>
+      <c r="F219" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152141.jpg</t>
+        </is>
+      </c>
+      <c r="G219" s="2" t="inlineStr">
+        <is>
+          <t>extra punches: 17:51 06:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B220" s="2" t="inlineStr">
+        <is>
+          <t>Employee 44</t>
+        </is>
+      </c>
+      <c r="C220" s="3" t="n">
+        <v>46254</v>
+      </c>
+      <c r="D220" s="4" t="n">
+        <v>0.7451388888888889</v>
+      </c>
+      <c r="E220" s="4" t="n">
+        <v>0.2583333333333334</v>
+      </c>
+      <c r="F220" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152141.jpg</t>
+        </is>
+      </c>
+      <c r="G220" s="2" t="inlineStr"/>
+    </row>
+    <row r="221">
+      <c r="A221" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B221" s="2" t="inlineStr">
+        <is>
+          <t>Employee 44</t>
+        </is>
+      </c>
+      <c r="C221" s="3" t="n">
+        <v>46253</v>
+      </c>
+      <c r="D221" s="4" t="n">
+        <v>0.7423611111111111</v>
+      </c>
+      <c r="E221" s="4" t="n">
+        <v>0.2527777777777778</v>
+      </c>
+      <c r="F221" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152141.jpg</t>
+        </is>
+      </c>
+      <c r="G221" s="2" t="inlineStr"/>
+    </row>
+    <row r="222">
+      <c r="A222" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B222" s="2" t="inlineStr">
+        <is>
+          <t>Employee 44</t>
+        </is>
+      </c>
+      <c r="C222" s="3" t="n">
+        <v>46252</v>
+      </c>
+      <c r="D222" s="4" t="n">
+        <v>0.7611111111111111</v>
+      </c>
+      <c r="E222" s="4" t="n">
+        <v>0.2395833333333333</v>
+      </c>
+      <c r="F222" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152141.jpg</t>
+        </is>
+      </c>
+      <c r="G222" s="2" t="inlineStr"/>
+    </row>
+    <row r="223">
+      <c r="A223" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B223" s="2" t="inlineStr">
+        <is>
+          <t>Employee 44</t>
+        </is>
+      </c>
+      <c r="C223" s="3" t="n">
+        <v>46251</v>
+      </c>
+      <c r="D223" s="4" t="n">
+        <v>0.7555555555555555</v>
+      </c>
+      <c r="E223" s="4" t="n">
+        <v>0.2541666666666667</v>
+      </c>
+      <c r="F223" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152158.jpg</t>
+        </is>
+      </c>
+      <c r="G223" s="2" t="inlineStr"/>
+    </row>
+    <row r="224">
+      <c r="A224" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B224" s="2" t="inlineStr">
+        <is>
+          <t>Employee 44</t>
+        </is>
+      </c>
+      <c r="C224" s="3" t="n">
+        <v>46250</v>
+      </c>
+      <c r="D224" s="4" t="n">
+        <v>0.7458333333333333</v>
+      </c>
+      <c r="E224" s="4" t="n">
+        <v>0.25625</v>
+      </c>
+      <c r="F224" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152158.jpg</t>
+        </is>
+      </c>
+      <c r="G224" s="2" t="inlineStr"/>
+    </row>
+    <row r="225">
+      <c r="A225" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B225" s="2" t="inlineStr">
+        <is>
+          <t>Employee 44</t>
+        </is>
+      </c>
+      <c r="C225" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="D225" s="4" t="n">
+        <v>0.7506944444444444</v>
+      </c>
+      <c r="E225" s="4" t="n">
+        <v>0.2333333333333333</v>
+      </c>
+      <c r="F225" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152158.jpg</t>
+        </is>
+      </c>
+      <c r="G225" s="2" t="inlineStr">
+        <is>
+          <t>extra punch: 06:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B226" s="2" t="inlineStr">
+        <is>
+          <t>Employee 44</t>
+        </is>
+      </c>
+      <c r="C226" s="3" t="n">
+        <v>46247</v>
+      </c>
+      <c r="D226" s="4" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E226" s="4" t="n">
+        <v>0.25625</v>
+      </c>
+      <c r="F226" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152158.jpg</t>
+        </is>
+      </c>
+      <c r="G226" s="2" t="inlineStr"/>
+    </row>
+    <row r="227">
+      <c r="A227" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B227" s="2" t="inlineStr">
+        <is>
+          <t>Employee 44</t>
+        </is>
+      </c>
+      <c r="C227" s="3" t="n">
+        <v>46246</v>
+      </c>
+      <c r="D227" s="4" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E227" s="4" t="n">
+        <v>0.2618055555555556</v>
+      </c>
+      <c r="F227" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152205.jpg</t>
+        </is>
+      </c>
+      <c r="G227" s="2" t="inlineStr"/>
+    </row>
+    <row r="228">
+      <c r="A228" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B228" s="2" t="inlineStr">
+        <is>
+          <t>Employee 44</t>
+        </is>
+      </c>
+      <c r="C228" s="3" t="n">
+        <v>46245</v>
+      </c>
+      <c r="D228" s="4" t="n">
+        <v>0.7465277777777778</v>
+      </c>
+      <c r="E228" s="4" t="n">
+        <v>0.2541666666666667</v>
+      </c>
+      <c r="F228" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152205.jpg</t>
+        </is>
+      </c>
+      <c r="G228" s="2" t="inlineStr"/>
+    </row>
+    <row r="229">
+      <c r="A229" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B229" s="2" t="inlineStr">
+        <is>
+          <t>Employee 44</t>
+        </is>
+      </c>
+      <c r="C229" s="3" t="n">
+        <v>46244</v>
+      </c>
+      <c r="D229" s="4" t="n">
+        <v>0.7479166666666667</v>
+      </c>
+      <c r="E229" s="4" t="n">
+        <v>0.2534722222222222</v>
+      </c>
+      <c r="F229" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152205.jpg</t>
+        </is>
+      </c>
+      <c r="G229" s="2" t="inlineStr"/>
+    </row>
+    <row r="230">
+      <c r="A230" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B230" s="2" t="inlineStr">
+        <is>
+          <t>Employee 44</t>
+        </is>
+      </c>
+      <c r="C230" s="3" t="n">
+        <v>46243</v>
+      </c>
+      <c r="D230" s="4" t="n">
+        <v>0.6729166666666667</v>
+      </c>
+      <c r="E230" s="4" t="n">
+        <v>0.2368055555555555</v>
+      </c>
+      <c r="F230" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152205.jpg</t>
+        </is>
+      </c>
+      <c r="G230" s="2" t="inlineStr"/>
+    </row>
+    <row r="231">
+      <c r="A231" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B231" s="2" t="inlineStr">
+        <is>
+          <t>Employee 44</t>
+        </is>
+      </c>
+      <c r="C231" s="3" t="n">
+        <v>46242</v>
+      </c>
+      <c r="D231" s="4" t="n">
+        <v>0.7291666666666666</v>
+      </c>
+      <c r="E231" s="4" t="n">
+        <v>0.2479166666666667</v>
+      </c>
+      <c r="F231" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152209.jpg</t>
+        </is>
+      </c>
+      <c r="G231" s="2" t="inlineStr">
+        <is>
+          <t>extra punch: 07:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B232" s="2" t="inlineStr">
+        <is>
+          <t>Employee 44</t>
+        </is>
+      </c>
+      <c r="C232" s="3" t="n">
+        <v>46240</v>
+      </c>
+      <c r="D232" s="4" t="n">
+        <v>0.75625</v>
+      </c>
+      <c r="E232" s="4" t="n">
+        <v>0.2277777777777778</v>
+      </c>
+      <c r="F232" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152209.jpg</t>
+        </is>
+      </c>
+      <c r="G232" s="2" t="inlineStr"/>
+    </row>
+    <row r="233">
+      <c r="A233" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B233" s="2" t="inlineStr">
+        <is>
+          <t>Employee 44</t>
+        </is>
+      </c>
+      <c r="C233" s="3" t="n">
+        <v>46239</v>
+      </c>
+      <c r="D233" s="4" t="n">
+        <v>0.7611111111111111</v>
+      </c>
+      <c r="E233" s="4" t="n">
+        <v>0.2333333333333333</v>
+      </c>
+      <c r="F233" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152209.jpg</t>
+        </is>
+      </c>
+      <c r="G233" s="2" t="inlineStr">
+        <is>
+          <t>extra punch: 18:16</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B234" s="2" t="inlineStr">
+        <is>
+          <t>Employee 44</t>
+        </is>
+      </c>
+      <c r="C234" s="3" t="n">
+        <v>46238</v>
+      </c>
+      <c r="D234" s="4" t="n">
+        <v>0.7604166666666666</v>
+      </c>
+      <c r="E234" s="4" t="n">
+        <v>0.2173611111111111</v>
+      </c>
+      <c r="F234" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152209.jpg</t>
+        </is>
+      </c>
+      <c r="G234" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Extract punch data for remaining employees (folder 1 batch)
Completes all 80 uploaded images. Adds employees 4, 6, 7, 9, 10, 19,
21, 25, 27, 28, plus fills gaps found for 37 and 41 from later
duplicate re-scans in the album, and corrects 6 employees' Aug 31
entries where the first pass had misread a two-punch day as a single
punch.

287 punch records total across 19 employees. 7 rows are flagged
"PLEASE VERIFY" in the notes column where a photo gap left a
check-in/out time unrecoverable, or a reading was ambiguous.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PeUzxoX8Admt6BxLMC3Cdz
</commit_message>
<xml_diff>
--- a/output/timesheet.xlsx
+++ b/output/timesheet.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G234"/>
+  <dimension ref="A1:G288"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1242,7 +1242,9 @@
       <c r="C29" s="3" t="n">
         <v>46265</v>
       </c>
-      <c r="D29" s="2" t="n"/>
+      <c r="D29" s="4" t="n">
+        <v>0.7354166666666667</v>
+      </c>
       <c r="E29" s="4" t="n">
         <v>0.2527777777777778</v>
       </c>
@@ -1253,7 +1255,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>single punch only</t>
+          <t>corrected from a clearer re-scan photo later in the album</t>
         </is>
       </c>
     </row>
@@ -2616,7 +2618,9 @@
       <c r="C79" s="3" t="n">
         <v>46265</v>
       </c>
-      <c r="D79" s="2" t="n"/>
+      <c r="D79" s="4" t="n">
+        <v>0.7604166666666666</v>
+      </c>
       <c r="E79" s="4" t="n">
         <v>0.2527777777777778</v>
       </c>
@@ -2627,7 +2631,7 @@
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>single punch only</t>
+          <t>corrected from a clearer re-scan photo later in the album</t>
         </is>
       </c>
     </row>
@@ -3363,7 +3367,9 @@
       <c r="C106" s="3" t="n">
         <v>46265</v>
       </c>
-      <c r="D106" s="2" t="n"/>
+      <c r="D106" s="4" t="n">
+        <v>0.7513888888888889</v>
+      </c>
       <c r="E106" s="4" t="n">
         <v>0.2777777777777778</v>
       </c>
@@ -3374,7 +3380,7 @@
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>single punch only</t>
+          <t>corrected from a clearer re-scan photo later in the album</t>
         </is>
       </c>
     </row>
@@ -4135,9 +4141,11 @@
       <c r="C134" s="3" t="n">
         <v>46265</v>
       </c>
-      <c r="D134" s="2" t="n"/>
+      <c r="D134" s="4" t="n">
+        <v>0.7520833333333333</v>
+      </c>
       <c r="E134" s="4" t="n">
-        <v>0.2416666666666667</v>
+        <v>0.2361111111111111</v>
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
@@ -4146,7 +4154,7 @@
       </c>
       <c r="G134" s="2" t="inlineStr">
         <is>
-          <t>single punch only</t>
+          <t>corrected from a clearer re-scan photo later in the album</t>
         </is>
       </c>
     </row>
@@ -5501,7 +5509,9 @@
       <c r="C184" s="3" t="n">
         <v>46265</v>
       </c>
-      <c r="D184" s="2" t="n"/>
+      <c r="D184" s="4" t="n">
+        <v>0.7215277777777778</v>
+      </c>
       <c r="E184" s="4" t="n">
         <v>0.3888888888888889</v>
       </c>
@@ -5512,7 +5522,7 @@
       </c>
       <c r="G184" s="2" t="inlineStr">
         <is>
-          <t>single punch only</t>
+          <t>corrected from a clearer re-scan photo later in the album</t>
         </is>
       </c>
     </row>
@@ -6266,7 +6276,9 @@
       <c r="C211" s="3" t="n">
         <v>46265</v>
       </c>
-      <c r="D211" s="2" t="n"/>
+      <c r="D211" s="4" t="n">
+        <v>0.7527777777777778</v>
+      </c>
       <c r="E211" s="4" t="n">
         <v>0.2569444444444444</v>
       </c>
@@ -6277,7 +6289,7 @@
       </c>
       <c r="G211" s="2" t="inlineStr">
         <is>
-          <t>single punch only</t>
+          <t>corrected from a clearer re-scan photo later in the album</t>
         </is>
       </c>
     </row>
@@ -6925,6 +6937,1490 @@
         </is>
       </c>
       <c r="G234" s="2" t="inlineStr"/>
+    </row>
+    <row r="235">
+      <c r="A235" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B235" s="2" t="inlineStr">
+        <is>
+          <t>Employee 44</t>
+        </is>
+      </c>
+      <c r="C235" s="3" t="n">
+        <v>46237</v>
+      </c>
+      <c r="D235" s="4" t="n">
+        <v>0.7402777777777778</v>
+      </c>
+      <c r="E235" s="4" t="n">
+        <v>0.2472222222222222</v>
+      </c>
+      <c r="F235" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152214.jpg</t>
+        </is>
+      </c>
+      <c r="G235" s="2" t="inlineStr">
+        <is>
+          <t>extra punch: 17:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B236" s="2" t="inlineStr">
+        <is>
+          <t>Employee 44</t>
+        </is>
+      </c>
+      <c r="C236" s="3" t="n">
+        <v>46236</v>
+      </c>
+      <c r="D236" s="4" t="n">
+        <v>0.7381944444444445</v>
+      </c>
+      <c r="E236" s="4" t="n">
+        <v>0.2201388888888889</v>
+      </c>
+      <c r="F236" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152214.jpg</t>
+        </is>
+      </c>
+      <c r="G236" s="2" t="inlineStr"/>
+    </row>
+    <row r="237">
+      <c r="A237" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B237" s="2" t="inlineStr">
+        <is>
+          <t>Employee 44</t>
+        </is>
+      </c>
+      <c r="C237" s="3" t="n">
+        <v>46235</v>
+      </c>
+      <c r="D237" s="4" t="n">
+        <v>0.7430555555555556</v>
+      </c>
+      <c r="E237" s="4" t="n">
+        <v>0.2569444444444444</v>
+      </c>
+      <c r="F237" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260831_152214.jpg</t>
+        </is>
+      </c>
+      <c r="G237" s="2" t="inlineStr">
+        <is>
+          <t>extra punch: 17:55; last day of month; final record</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B238" s="2" t="inlineStr">
+        <is>
+          <t>Employee 4</t>
+        </is>
+      </c>
+      <c r="C238" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="D238" s="4" t="n">
+        <v>0.7527777777777778</v>
+      </c>
+      <c r="E238" s="4" t="n">
+        <v>0.2493055555555556</v>
+      </c>
+      <c r="F238" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_065955.jpg</t>
+        </is>
+      </c>
+      <c r="G238" s="2" t="inlineStr"/>
+    </row>
+    <row r="239">
+      <c r="A239" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B239" s="2" t="inlineStr">
+        <is>
+          <t>Employee 4</t>
+        </is>
+      </c>
+      <c r="C239" s="3" t="n">
+        <v>46264</v>
+      </c>
+      <c r="D239" s="4" t="n">
+        <v>0.7458333333333333</v>
+      </c>
+      <c r="E239" s="4" t="n">
+        <v>0.3006944444444444</v>
+      </c>
+      <c r="F239" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_065955.jpg</t>
+        </is>
+      </c>
+      <c r="G239" s="2" t="inlineStr"/>
+    </row>
+    <row r="240">
+      <c r="A240" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B240" s="2" t="inlineStr">
+        <is>
+          <t>Employee 4</t>
+        </is>
+      </c>
+      <c r="C240" s="3" t="n">
+        <v>46263</v>
+      </c>
+      <c r="D240" s="4" t="n">
+        <v>0.6736111111111112</v>
+      </c>
+      <c r="E240" s="4" t="n">
+        <v>0.30625</v>
+      </c>
+      <c r="F240" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_065955.jpg</t>
+        </is>
+      </c>
+      <c r="G240" s="2" t="inlineStr"/>
+    </row>
+    <row r="241">
+      <c r="A241" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B241" s="2" t="inlineStr">
+        <is>
+          <t>Employee 4</t>
+        </is>
+      </c>
+      <c r="C241" s="3" t="n">
+        <v>46261</v>
+      </c>
+      <c r="D241" s="4" t="n">
+        <v>0.6916666666666667</v>
+      </c>
+      <c r="E241" s="4" t="n">
+        <v>0.2791666666666667</v>
+      </c>
+      <c r="F241" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_065955.jpg</t>
+        </is>
+      </c>
+      <c r="G241" s="2" t="inlineStr"/>
+    </row>
+    <row r="242">
+      <c r="A242" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B242" s="2" t="inlineStr">
+        <is>
+          <t>Employee 4</t>
+        </is>
+      </c>
+      <c r="C242" s="3" t="n">
+        <v>46260</v>
+      </c>
+      <c r="D242" s="2" t="n"/>
+      <c r="E242" s="2" t="n"/>
+      <c r="F242" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_065955.jpg</t>
+        </is>
+      </c>
+      <c r="G242" s="2" t="inlineStr">
+        <is>
+          <t>PLEASE VERIFY: check-in/out times not captured (gap between source photos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B243" s="2" t="inlineStr">
+        <is>
+          <t>Employee 6</t>
+        </is>
+      </c>
+      <c r="C243" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="D243" s="4" t="n">
+        <v>0.7375</v>
+      </c>
+      <c r="E243" s="4" t="n">
+        <v>0.2451388888888889</v>
+      </c>
+      <c r="F243" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070012.jpg</t>
+        </is>
+      </c>
+      <c r="G243" s="2" t="inlineStr"/>
+    </row>
+    <row r="244">
+      <c r="A244" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B244" s="2" t="inlineStr">
+        <is>
+          <t>Employee 6</t>
+        </is>
+      </c>
+      <c r="C244" s="3" t="n">
+        <v>46264</v>
+      </c>
+      <c r="D244" s="4" t="n">
+        <v>0.6888888888888889</v>
+      </c>
+      <c r="E244" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F244" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070012.jpg</t>
+        </is>
+      </c>
+      <c r="G244" s="2" t="inlineStr"/>
+    </row>
+    <row r="245">
+      <c r="A245" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B245" s="2" t="inlineStr">
+        <is>
+          <t>Employee 6</t>
+        </is>
+      </c>
+      <c r="C245" s="3" t="n">
+        <v>46263</v>
+      </c>
+      <c r="D245" s="4" t="n">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="E245" s="4" t="n">
+        <v>0.2465277777777778</v>
+      </c>
+      <c r="F245" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070012.jpg</t>
+        </is>
+      </c>
+      <c r="G245" s="2" t="inlineStr"/>
+    </row>
+    <row r="246">
+      <c r="A246" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B246" s="2" t="inlineStr">
+        <is>
+          <t>Employee 6</t>
+        </is>
+      </c>
+      <c r="C246" s="3" t="n">
+        <v>46261</v>
+      </c>
+      <c r="D246" s="4" t="n">
+        <v>0.6986111111111111</v>
+      </c>
+      <c r="E246" s="4" t="n">
+        <v>0.2569444444444444</v>
+      </c>
+      <c r="F246" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070012.jpg</t>
+        </is>
+      </c>
+      <c r="G246" s="2" t="inlineStr"/>
+    </row>
+    <row r="247">
+      <c r="A247" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B247" s="2" t="inlineStr">
+        <is>
+          <t>Employee 6</t>
+        </is>
+      </c>
+      <c r="C247" s="3" t="n">
+        <v>46260</v>
+      </c>
+      <c r="D247" s="2" t="n"/>
+      <c r="E247" s="2" t="n"/>
+      <c r="F247" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070012.jpg</t>
+        </is>
+      </c>
+      <c r="G247" s="2" t="inlineStr">
+        <is>
+          <t>PLEASE VERIFY: check-in/out times not captured (gap between source photos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B248" s="2" t="inlineStr">
+        <is>
+          <t>Employee 7</t>
+        </is>
+      </c>
+      <c r="C248" s="3" t="n">
+        <v>46263</v>
+      </c>
+      <c r="D248" s="2" t="n"/>
+      <c r="E248" s="4" t="n">
+        <v>0.2986111111111111</v>
+      </c>
+      <c r="F248" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070022.jpg</t>
+        </is>
+      </c>
+      <c r="G248" s="2" t="inlineStr">
+        <is>
+          <t>single punch only</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B249" s="2" t="inlineStr">
+        <is>
+          <t>Employee 7</t>
+        </is>
+      </c>
+      <c r="C249" s="3" t="n">
+        <v>46261</v>
+      </c>
+      <c r="D249" s="4" t="n">
+        <v>0.8090277777777778</v>
+      </c>
+      <c r="E249" s="4" t="n">
+        <v>0.3375</v>
+      </c>
+      <c r="F249" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070022.jpg</t>
+        </is>
+      </c>
+      <c r="G249" s="2" t="inlineStr"/>
+    </row>
+    <row r="250">
+      <c r="A250" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B250" s="2" t="inlineStr">
+        <is>
+          <t>Employee 7</t>
+        </is>
+      </c>
+      <c r="C250" s="3" t="n">
+        <v>46260</v>
+      </c>
+      <c r="D250" s="4" t="n">
+        <v>0.8083333333333333</v>
+      </c>
+      <c r="E250" s="4" t="n">
+        <v>0.3854166666666667</v>
+      </c>
+      <c r="F250" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070022.jpg</t>
+        </is>
+      </c>
+      <c r="G250" s="2" t="inlineStr"/>
+    </row>
+    <row r="251">
+      <c r="A251" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B251" s="2" t="inlineStr">
+        <is>
+          <t>Employee 7</t>
+        </is>
+      </c>
+      <c r="C251" s="3" t="n">
+        <v>46259</v>
+      </c>
+      <c r="D251" s="4" t="n">
+        <v>0.7506944444444444</v>
+      </c>
+      <c r="E251" s="4" t="n">
+        <v>0.2673611111111111</v>
+      </c>
+      <c r="F251" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070022.jpg</t>
+        </is>
+      </c>
+      <c r="G251" s="2" t="inlineStr"/>
+    </row>
+    <row r="252">
+      <c r="A252" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B252" s="2" t="inlineStr">
+        <is>
+          <t>Employee 9</t>
+        </is>
+      </c>
+      <c r="C252" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="D252" s="4" t="n">
+        <v>0.7555555555555555</v>
+      </c>
+      <c r="E252" s="4" t="n">
+        <v>0.2472222222222222</v>
+      </c>
+      <c r="F252" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070037.jpg</t>
+        </is>
+      </c>
+      <c r="G252" s="2" t="inlineStr"/>
+    </row>
+    <row r="253">
+      <c r="A253" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B253" s="2" t="inlineStr">
+        <is>
+          <t>Employee 9</t>
+        </is>
+      </c>
+      <c r="C253" s="3" t="n">
+        <v>46264</v>
+      </c>
+      <c r="D253" s="4" t="n">
+        <v>0.6805555555555556</v>
+      </c>
+      <c r="E253" s="4" t="n">
+        <v>0.30625</v>
+      </c>
+      <c r="F253" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070037.jpg</t>
+        </is>
+      </c>
+      <c r="G253" s="2" t="inlineStr"/>
+    </row>
+    <row r="254">
+      <c r="A254" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B254" s="2" t="inlineStr">
+        <is>
+          <t>Employee 9</t>
+        </is>
+      </c>
+      <c r="C254" s="3" t="n">
+        <v>46263</v>
+      </c>
+      <c r="D254" s="4" t="n">
+        <v>0.7708333333333334</v>
+      </c>
+      <c r="E254" s="4" t="n">
+        <v>0.2993055555555555</v>
+      </c>
+      <c r="F254" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070037.jpg</t>
+        </is>
+      </c>
+      <c r="G254" s="2" t="inlineStr"/>
+    </row>
+    <row r="255">
+      <c r="A255" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B255" s="2" t="inlineStr">
+        <is>
+          <t>Employee 9</t>
+        </is>
+      </c>
+      <c r="C255" s="3" t="n">
+        <v>46261</v>
+      </c>
+      <c r="D255" s="4" t="n">
+        <v>0.7861111111111111</v>
+      </c>
+      <c r="E255" s="4" t="n">
+        <v>0.2826388888888889</v>
+      </c>
+      <c r="F255" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070037.jpg</t>
+        </is>
+      </c>
+      <c r="G255" s="2" t="inlineStr"/>
+    </row>
+    <row r="256">
+      <c r="A256" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B256" s="2" t="inlineStr">
+        <is>
+          <t>Employee 9</t>
+        </is>
+      </c>
+      <c r="C256" s="3" t="n">
+        <v>46260</v>
+      </c>
+      <c r="D256" s="2" t="n"/>
+      <c r="E256" s="2" t="n"/>
+      <c r="F256" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070037.jpg</t>
+        </is>
+      </c>
+      <c r="G256" s="2" t="inlineStr">
+        <is>
+          <t>PLEASE VERIFY: check-in/out times not captured (gap between source photos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B257" s="2" t="inlineStr">
+        <is>
+          <t>Employee 10</t>
+        </is>
+      </c>
+      <c r="C257" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="D257" s="4" t="n">
+        <v>0.7534722222222222</v>
+      </c>
+      <c r="E257" s="4" t="n">
+        <v>0.2805555555555556</v>
+      </c>
+      <c r="F257" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070045.jpg</t>
+        </is>
+      </c>
+      <c r="G257" s="2" t="inlineStr"/>
+    </row>
+    <row r="258">
+      <c r="A258" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B258" s="2" t="inlineStr">
+        <is>
+          <t>Employee 10</t>
+        </is>
+      </c>
+      <c r="C258" s="3" t="n">
+        <v>46263</v>
+      </c>
+      <c r="D258" s="4" t="n">
+        <v>0.4041666666666667</v>
+      </c>
+      <c r="E258" s="2" t="n"/>
+      <c r="F258" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070045.jpg</t>
+        </is>
+      </c>
+      <c r="G258" s="2" t="inlineStr">
+        <is>
+          <t>single punch only</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B259" s="2" t="inlineStr">
+        <is>
+          <t>Employee 10</t>
+        </is>
+      </c>
+      <c r="C259" s="3" t="n">
+        <v>46261</v>
+      </c>
+      <c r="D259" s="4" t="n">
+        <v>0.7395833333333334</v>
+      </c>
+      <c r="E259" s="2" t="n"/>
+      <c r="F259" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070045.jpg</t>
+        </is>
+      </c>
+      <c r="G259" s="2" t="inlineStr">
+        <is>
+          <t>single punch only</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B260" s="2" t="inlineStr">
+        <is>
+          <t>Employee 10</t>
+        </is>
+      </c>
+      <c r="C260" s="3" t="n">
+        <v>46259</v>
+      </c>
+      <c r="D260" s="4" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E260" s="2" t="n"/>
+      <c r="F260" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070045.jpg</t>
+        </is>
+      </c>
+      <c r="G260" s="2" t="inlineStr">
+        <is>
+          <t>single punch only</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B261" s="2" t="inlineStr">
+        <is>
+          <t>Employee 10</t>
+        </is>
+      </c>
+      <c r="C261" s="3" t="n">
+        <v>46258</v>
+      </c>
+      <c r="D261" s="2" t="n"/>
+      <c r="E261" s="2" t="n"/>
+      <c r="F261" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070045.jpg</t>
+        </is>
+      </c>
+      <c r="G261" s="2" t="inlineStr">
+        <is>
+          <t>PLEASE VERIFY: check-in/out time not captured (gap between source photos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="2" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B262" s="2" t="inlineStr">
+        <is>
+          <t>Employee 19</t>
+        </is>
+      </c>
+      <c r="C262" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="D262" s="4" t="n">
+        <v>0.7680555555555556</v>
+      </c>
+      <c r="E262" s="4" t="n">
+        <v>0.3319444444444444</v>
+      </c>
+      <c r="F262" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070157.jpg</t>
+        </is>
+      </c>
+      <c r="G262" s="2" t="inlineStr"/>
+    </row>
+    <row r="263">
+      <c r="A263" s="2" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B263" s="2" t="inlineStr">
+        <is>
+          <t>Employee 19</t>
+        </is>
+      </c>
+      <c r="C263" s="3" t="n">
+        <v>46264</v>
+      </c>
+      <c r="D263" s="4" t="n">
+        <v>0.7534722222222222</v>
+      </c>
+      <c r="E263" s="4" t="n">
+        <v>0.3534722222222222</v>
+      </c>
+      <c r="F263" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070157.jpg</t>
+        </is>
+      </c>
+      <c r="G263" s="2" t="inlineStr"/>
+    </row>
+    <row r="264">
+      <c r="A264" s="2" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B264" s="2" t="inlineStr">
+        <is>
+          <t>Employee 19</t>
+        </is>
+      </c>
+      <c r="C264" s="3" t="n">
+        <v>46263</v>
+      </c>
+      <c r="D264" s="4" t="n">
+        <v>0.7569444444444444</v>
+      </c>
+      <c r="E264" s="4" t="n">
+        <v>0.3652777777777778</v>
+      </c>
+      <c r="F264" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070157.jpg</t>
+        </is>
+      </c>
+      <c r="G264" s="2" t="inlineStr"/>
+    </row>
+    <row r="265">
+      <c r="A265" s="2" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B265" s="2" t="inlineStr">
+        <is>
+          <t>Employee 19</t>
+        </is>
+      </c>
+      <c r="C265" s="3" t="n">
+        <v>46261</v>
+      </c>
+      <c r="D265" s="4" t="n">
+        <v>0.7395833333333334</v>
+      </c>
+      <c r="E265" s="4" t="n">
+        <v>0.3652777777777778</v>
+      </c>
+      <c r="F265" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070157.jpg</t>
+        </is>
+      </c>
+      <c r="G265" s="2" t="inlineStr"/>
+    </row>
+    <row r="266">
+      <c r="A266" s="2" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B266" s="2" t="inlineStr">
+        <is>
+          <t>Employee 19</t>
+        </is>
+      </c>
+      <c r="C266" s="3" t="n">
+        <v>46260</v>
+      </c>
+      <c r="D266" s="2" t="n"/>
+      <c r="E266" s="2" t="n"/>
+      <c r="F266" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070157.jpg</t>
+        </is>
+      </c>
+      <c r="G266" s="2" t="inlineStr">
+        <is>
+          <t>PLEASE VERIFY: check-in/out times not captured (gap between source photos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="2" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B267" s="2" t="inlineStr">
+        <is>
+          <t>Employee 21</t>
+        </is>
+      </c>
+      <c r="C267" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="D267" s="4" t="n">
+        <v>0.7555555555555555</v>
+      </c>
+      <c r="E267" s="4" t="n">
+        <v>0.2631944444444445</v>
+      </c>
+      <c r="F267" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070210.jpg</t>
+        </is>
+      </c>
+      <c r="G267" s="2" t="inlineStr"/>
+    </row>
+    <row r="268">
+      <c r="A268" s="2" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B268" s="2" t="inlineStr">
+        <is>
+          <t>Employee 21</t>
+        </is>
+      </c>
+      <c r="C268" s="3" t="n">
+        <v>46264</v>
+      </c>
+      <c r="D268" s="4" t="n">
+        <v>0.7493055555555556</v>
+      </c>
+      <c r="E268" s="4" t="n">
+        <v>0.3194444444444444</v>
+      </c>
+      <c r="F268" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070210.jpg</t>
+        </is>
+      </c>
+      <c r="G268" s="2" t="inlineStr"/>
+    </row>
+    <row r="269">
+      <c r="A269" s="2" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B269" s="2" t="inlineStr">
+        <is>
+          <t>Employee 21</t>
+        </is>
+      </c>
+      <c r="C269" s="3" t="n">
+        <v>46263</v>
+      </c>
+      <c r="D269" s="4" t="n">
+        <v>0.7513888888888889</v>
+      </c>
+      <c r="E269" s="4" t="n">
+        <v>0.275</v>
+      </c>
+      <c r="F269" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070210.jpg</t>
+        </is>
+      </c>
+      <c r="G269" s="2" t="inlineStr"/>
+    </row>
+    <row r="270">
+      <c r="A270" s="2" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B270" s="2" t="inlineStr">
+        <is>
+          <t>Employee 21</t>
+        </is>
+      </c>
+      <c r="C270" s="3" t="n">
+        <v>46261</v>
+      </c>
+      <c r="D270" s="4" t="n">
+        <v>0.7430555555555556</v>
+      </c>
+      <c r="E270" s="4" t="n">
+        <v>0.2909722222222222</v>
+      </c>
+      <c r="F270" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070210.jpg</t>
+        </is>
+      </c>
+      <c r="G270" s="2" t="inlineStr"/>
+    </row>
+    <row r="271">
+      <c r="A271" s="2" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B271" s="2" t="inlineStr">
+        <is>
+          <t>Employee 21</t>
+        </is>
+      </c>
+      <c r="C271" s="3" t="n">
+        <v>46260</v>
+      </c>
+      <c r="D271" s="2" t="n"/>
+      <c r="E271" s="2" t="n"/>
+      <c r="F271" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070210.jpg</t>
+        </is>
+      </c>
+      <c r="G271" s="2" t="inlineStr">
+        <is>
+          <t>PLEASE VERIFY: check-in/out times not captured (gap between source photos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="2" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="B272" s="2" t="inlineStr">
+        <is>
+          <t>Employee 25</t>
+        </is>
+      </c>
+      <c r="C272" s="3" t="n">
+        <v>46264</v>
+      </c>
+      <c r="D272" s="4" t="n">
+        <v>0.7354166666666667</v>
+      </c>
+      <c r="E272" s="4" t="n">
+        <v>0.3208333333333334</v>
+      </c>
+      <c r="F272" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070242.jpg</t>
+        </is>
+      </c>
+      <c r="G272" s="2" t="inlineStr"/>
+    </row>
+    <row r="273">
+      <c r="A273" s="2" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="B273" s="2" t="inlineStr">
+        <is>
+          <t>Employee 25</t>
+        </is>
+      </c>
+      <c r="C273" s="3" t="n">
+        <v>46263</v>
+      </c>
+      <c r="D273" s="4" t="n">
+        <v>0.8895833333333333</v>
+      </c>
+      <c r="E273" s="4" t="n">
+        <v>0.3347222222222222</v>
+      </c>
+      <c r="F273" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070242.jpg</t>
+        </is>
+      </c>
+      <c r="G273" s="2" t="inlineStr">
+        <is>
+          <t>extra punch: 08:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="2" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="B274" s="2" t="inlineStr">
+        <is>
+          <t>Employee 25</t>
+        </is>
+      </c>
+      <c r="C274" s="3" t="n">
+        <v>46261</v>
+      </c>
+      <c r="D274" s="4" t="n">
+        <v>0.7493055555555556</v>
+      </c>
+      <c r="E274" s="4" t="n">
+        <v>0.2798611111111111</v>
+      </c>
+      <c r="F274" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070242.jpg</t>
+        </is>
+      </c>
+      <c r="G274" s="2" t="inlineStr"/>
+    </row>
+    <row r="275">
+      <c r="A275" s="2" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="B275" s="2" t="inlineStr">
+        <is>
+          <t>Employee 25</t>
+        </is>
+      </c>
+      <c r="C275" s="3" t="n">
+        <v>46260</v>
+      </c>
+      <c r="D275" s="4" t="n">
+        <v>0.8013888888888889</v>
+      </c>
+      <c r="E275" s="4" t="n">
+        <v>0.3055555555555556</v>
+      </c>
+      <c r="F275" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070242.jpg</t>
+        </is>
+      </c>
+      <c r="G275" s="2" t="inlineStr"/>
+    </row>
+    <row r="276">
+      <c r="A276" s="2" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="B276" s="2" t="inlineStr">
+        <is>
+          <t>Employee 27</t>
+        </is>
+      </c>
+      <c r="C276" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="D276" s="4" t="n">
+        <v>0.9326388888888889</v>
+      </c>
+      <c r="E276" s="4" t="n">
+        <v>0.1479166666666667</v>
+      </c>
+      <c r="F276" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070256.jpg</t>
+        </is>
+      </c>
+      <c r="G276" s="2" t="inlineStr">
+        <is>
+          <t>extra punch: 22:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="2" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="B277" s="2" t="inlineStr">
+        <is>
+          <t>Employee 27</t>
+        </is>
+      </c>
+      <c r="C277" s="3" t="n">
+        <v>46264</v>
+      </c>
+      <c r="D277" s="4" t="n">
+        <v>0.75625</v>
+      </c>
+      <c r="E277" s="4" t="n">
+        <v>0.14375</v>
+      </c>
+      <c r="F277" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070256.jpg</t>
+        </is>
+      </c>
+      <c r="G277" s="2" t="inlineStr"/>
+    </row>
+    <row r="278">
+      <c r="A278" s="2" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="B278" s="2" t="inlineStr">
+        <is>
+          <t>Employee 27</t>
+        </is>
+      </c>
+      <c r="C278" s="3" t="n">
+        <v>46263</v>
+      </c>
+      <c r="D278" s="4" t="n">
+        <v>0.7479166666666667</v>
+      </c>
+      <c r="E278" s="4" t="n">
+        <v>0.1451388888888889</v>
+      </c>
+      <c r="F278" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070256.jpg</t>
+        </is>
+      </c>
+      <c r="G278" s="2" t="inlineStr"/>
+    </row>
+    <row r="279">
+      <c r="A279" s="2" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="B279" s="2" t="inlineStr">
+        <is>
+          <t>Employee 27</t>
+        </is>
+      </c>
+      <c r="C279" s="3" t="n">
+        <v>46262</v>
+      </c>
+      <c r="D279" s="4" t="n">
+        <v>0.7159722222222222</v>
+      </c>
+      <c r="E279" s="4" t="n">
+        <v>0.1493055555555556</v>
+      </c>
+      <c r="F279" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070256.jpg</t>
+        </is>
+      </c>
+      <c r="G279" s="2" t="inlineStr"/>
+    </row>
+    <row r="280">
+      <c r="A280" s="2" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="B280" s="2" t="inlineStr">
+        <is>
+          <t>Employee 28</t>
+        </is>
+      </c>
+      <c r="C280" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="D280" s="4" t="n">
+        <v>0.4131944444444444</v>
+      </c>
+      <c r="E280" s="4" t="n">
+        <v>0.1868055555555556</v>
+      </c>
+      <c r="F280" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070305.jpg</t>
+        </is>
+      </c>
+      <c r="G280" s="2" t="inlineStr"/>
+    </row>
+    <row r="281">
+      <c r="A281" s="2" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="B281" s="2" t="inlineStr">
+        <is>
+          <t>Employee 28</t>
+        </is>
+      </c>
+      <c r="C281" s="3" t="n">
+        <v>46264</v>
+      </c>
+      <c r="D281" s="4" t="n">
+        <v>0.5097222222222222</v>
+      </c>
+      <c r="E281" s="4" t="n">
+        <v>0.1847222222222222</v>
+      </c>
+      <c r="F281" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070305.jpg</t>
+        </is>
+      </c>
+      <c r="G281" s="2" t="inlineStr"/>
+    </row>
+    <row r="282">
+      <c r="A282" s="2" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="B282" s="2" t="inlineStr">
+        <is>
+          <t>Employee 28</t>
+        </is>
+      </c>
+      <c r="C282" s="3" t="n">
+        <v>46263</v>
+      </c>
+      <c r="D282" s="4" t="n">
+        <v>0.4527777777777778</v>
+      </c>
+      <c r="E282" s="4" t="n">
+        <v>0.1847222222222222</v>
+      </c>
+      <c r="F282" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070305.jpg</t>
+        </is>
+      </c>
+      <c r="G282" s="2" t="inlineStr"/>
+    </row>
+    <row r="283">
+      <c r="A283" s="2" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="B283" s="2" t="inlineStr">
+        <is>
+          <t>Employee 28</t>
+        </is>
+      </c>
+      <c r="C283" s="3" t="n">
+        <v>46262</v>
+      </c>
+      <c r="D283" s="4" t="n">
+        <v>0.4055555555555556</v>
+      </c>
+      <c r="E283" s="4" t="n">
+        <v>0.1881944444444444</v>
+      </c>
+      <c r="F283" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070305.jpg</t>
+        </is>
+      </c>
+      <c r="G283" s="2" t="inlineStr"/>
+    </row>
+    <row r="284">
+      <c r="A284" s="2" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="B284" s="2" t="inlineStr">
+        <is>
+          <t>Employee 37</t>
+        </is>
+      </c>
+      <c r="C284" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="D284" s="4" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E284" s="4" t="n">
+        <v>0.2909722222222222</v>
+      </c>
+      <c r="F284" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070423.jpg</t>
+        </is>
+      </c>
+      <c r="G284" s="2" t="inlineStr"/>
+    </row>
+    <row r="285">
+      <c r="A285" s="2" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="B285" s="2" t="inlineStr">
+        <is>
+          <t>Employee 37</t>
+        </is>
+      </c>
+      <c r="C285" s="3" t="n">
+        <v>46264</v>
+      </c>
+      <c r="D285" s="4" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E285" s="4" t="n">
+        <v>0.2888888888888889</v>
+      </c>
+      <c r="F285" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070423.jpg</t>
+        </is>
+      </c>
+      <c r="G285" s="2" t="inlineStr"/>
+    </row>
+    <row r="286">
+      <c r="A286" s="2" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="B286" s="2" t="inlineStr">
+        <is>
+          <t>Employee 37</t>
+        </is>
+      </c>
+      <c r="C286" s="3" t="n">
+        <v>46263</v>
+      </c>
+      <c r="D286" s="4" t="n">
+        <v>0.7472222222222222</v>
+      </c>
+      <c r="E286" s="4" t="n">
+        <v>0.2965277777777778</v>
+      </c>
+      <c r="F286" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070423.jpg</t>
+        </is>
+      </c>
+      <c r="G286" s="2" t="inlineStr"/>
+    </row>
+    <row r="287">
+      <c r="A287" s="2" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="B287" s="2" t="inlineStr">
+        <is>
+          <t>Employee 37</t>
+        </is>
+      </c>
+      <c r="C287" s="3" t="n">
+        <v>46261</v>
+      </c>
+      <c r="D287" s="4" t="n">
+        <v>0.6763888888888889</v>
+      </c>
+      <c r="E287" s="4" t="n">
+        <v>0.24375</v>
+      </c>
+      <c r="F287" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070423.jpg</t>
+        </is>
+      </c>
+      <c r="G287" s="2" t="inlineStr"/>
+    </row>
+    <row r="288">
+      <c r="A288" s="2" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B288" s="2" t="inlineStr">
+        <is>
+          <t>Employee 41</t>
+        </is>
+      </c>
+      <c r="C288" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="D288" s="4" t="n">
+        <v>0.7097222222222223</v>
+      </c>
+      <c r="E288" s="2" t="n"/>
+      <c r="F288" s="2" t="inlineStr">
+        <is>
+          <t>IMG_20260901_070506.jpg</t>
+        </is>
+      </c>
+      <c r="G288" s="2" t="inlineStr">
+        <is>
+          <t>single punch only</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Label employee 25 as Night Security
Employee 25's shift pattern (evening check-in, early-morning checkout)
is confirmed to be an overnight security shift. Tagged "Night Security"
in the notes field for all 28 of their records.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PeUzxoX8Admt6BxLMC3Cdz
</commit_message>
<xml_diff>
--- a/output/timesheet.xlsx
+++ b/output/timesheet.xlsx
@@ -4460,7 +4460,7 @@
       </c>
       <c r="E195" s="2" t="inlineStr">
         <is>
-          <t>single punch only; last day of month</t>
+          <t>Night Security; single punch only; last day of month</t>
         </is>
       </c>
     </row>
@@ -4483,7 +4483,7 @@
       </c>
       <c r="E196" s="2" t="inlineStr">
         <is>
-          <t>single punch only</t>
+          <t>Night Security; single punch only</t>
         </is>
       </c>
     </row>
@@ -4504,7 +4504,7 @@
       </c>
       <c r="E197" s="2" t="inlineStr">
         <is>
-          <t>extra punch: 17:50</t>
+          <t>Night Security; extra punch: 17:50</t>
         </is>
       </c>
     </row>
@@ -4525,7 +4525,7 @@
       </c>
       <c r="E198" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Night Security</t>
         </is>
       </c>
     </row>
@@ -4548,7 +4548,7 @@
       </c>
       <c r="E199" s="2" t="inlineStr">
         <is>
-          <t>single punch only</t>
+          <t>Night Security; single punch only</t>
         </is>
       </c>
     </row>
@@ -4569,7 +4569,7 @@
       </c>
       <c r="E200" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Night Security</t>
         </is>
       </c>
     </row>
@@ -4592,7 +4592,7 @@
       </c>
       <c r="E201" s="2" t="inlineStr">
         <is>
-          <t>single punch only</t>
+          <t>Night Security; single punch only</t>
         </is>
       </c>
     </row>
@@ -4613,7 +4613,7 @@
       </c>
       <c r="E202" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Night Security</t>
         </is>
       </c>
     </row>
@@ -4634,7 +4634,7 @@
       </c>
       <c r="E203" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Night Security</t>
         </is>
       </c>
     </row>
@@ -4657,7 +4657,7 @@
       </c>
       <c r="E204" s="2" t="inlineStr">
         <is>
-          <t>single punch only</t>
+          <t>Night Security; single punch only</t>
         </is>
       </c>
     </row>
@@ -4678,7 +4678,7 @@
       </c>
       <c r="E205" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Night Security</t>
         </is>
       </c>
     </row>
@@ -4699,7 +4699,7 @@
       </c>
       <c r="E206" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Night Security</t>
         </is>
       </c>
     </row>
@@ -4720,7 +4720,7 @@
       </c>
       <c r="E207" s="2" t="inlineStr">
         <is>
-          <t>PLEASE VERIFY: extra punches 05:39 05:39 05:39 05:39 repeated - possible device anomaly</t>
+          <t>Night Security; PLEASE VERIFY: extra punches 05:39 05:39 05:39 05:39 repeated - possible device anomaly</t>
         </is>
       </c>
     </row>
@@ -4741,7 +4741,7 @@
       </c>
       <c r="E208" s="2" t="inlineStr">
         <is>
-          <t>extra punch: 09:31</t>
+          <t>Night Security; extra punch: 09:31</t>
         </is>
       </c>
     </row>
@@ -4764,7 +4764,7 @@
       </c>
       <c r="E209" s="2" t="inlineStr">
         <is>
-          <t>single punch only</t>
+          <t>Night Security; single punch only</t>
         </is>
       </c>
     </row>
@@ -4785,7 +4785,7 @@
       </c>
       <c r="E210" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Night Security</t>
         </is>
       </c>
     </row>
@@ -4806,7 +4806,7 @@
       </c>
       <c r="E211" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Night Security</t>
         </is>
       </c>
     </row>
@@ -4827,7 +4827,7 @@
       </c>
       <c r="E212" s="2" t="inlineStr">
         <is>
-          <t>extra punch: 17:19</t>
+          <t>Night Security; extra punch: 17:19</t>
         </is>
       </c>
     </row>
@@ -4850,7 +4850,7 @@
       </c>
       <c r="E213" s="2" t="inlineStr">
         <is>
-          <t>single punch only</t>
+          <t>Night Security; single punch only</t>
         </is>
       </c>
     </row>
@@ -4871,7 +4871,7 @@
       </c>
       <c r="E214" s="2" t="inlineStr">
         <is>
-          <t>PLEASE VERIFY: in/out times read identical - likely OCR error</t>
+          <t>Night Security; PLEASE VERIFY: in/out times read identical - likely OCR error</t>
         </is>
       </c>
     </row>
@@ -4892,7 +4892,7 @@
       </c>
       <c r="E215" s="2" t="inlineStr">
         <is>
-          <t>extra punch: 05:45</t>
+          <t>Night Security; extra punch: 05:45</t>
         </is>
       </c>
     </row>
@@ -4913,7 +4913,7 @@
       </c>
       <c r="E216" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Night Security</t>
         </is>
       </c>
     </row>
@@ -4934,7 +4934,7 @@
       </c>
       <c r="E217" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Night Security</t>
         </is>
       </c>
     </row>
@@ -4955,7 +4955,7 @@
       </c>
       <c r="E218" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Night Security</t>
         </is>
       </c>
     </row>
@@ -4976,7 +4976,7 @@
       </c>
       <c r="E219" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Night Security</t>
         </is>
       </c>
     </row>
@@ -4997,7 +4997,7 @@
       </c>
       <c r="E220" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Night Security</t>
         </is>
       </c>
     </row>
@@ -5018,7 +5018,7 @@
       </c>
       <c r="E221" s="2" t="inlineStr">
         <is>
-          <t>extra punch: 08:02</t>
+          <t>Night Security; extra punch: 08:02</t>
         </is>
       </c>
     </row>
@@ -5039,7 +5039,7 @@
       </c>
       <c r="E222" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Night Security</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Highlight Friday rows in yellow
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PeUzxoX8Admt6BxLMC3Cdz
</commit_message>
<xml_diff>
--- a/output/timesheet.xlsx
+++ b/output/timesheet.xlsx
@@ -37,7 +37,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -48,6 +48,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="001F4E78"/>
         <bgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -63,7 +69,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -71,6 +77,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2988,23 +2997,23 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="2" t="inlineStr">
+      <c r="A124" s="5" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B124" s="3" t="n">
+      <c r="B124" s="6" t="n">
         <v>46248</v>
       </c>
-      <c r="C124" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D124" s="4" t="n">
+      <c r="C124" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D124" s="7" t="n">
         <v>0.7708333333333334</v>
       </c>
-      <c r="E124" s="2" t="inlineStr">
+      <c r="E124" s="5" t="inlineStr">
         <is>
           <t>single punch only</t>
         </is>
@@ -3147,23 +3156,23 @@
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="2" t="inlineStr">
+      <c r="A131" s="5" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B131" s="3" t="n">
+      <c r="B131" s="6" t="n">
         <v>46255</v>
       </c>
-      <c r="C131" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D131" s="4" t="n">
+      <c r="C131" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D131" s="7" t="n">
         <v>0.7333333333333333</v>
       </c>
-      <c r="E131" s="2" t="inlineStr">
+      <c r="E131" s="5" t="inlineStr">
         <is>
           <t>single punch only</t>
         </is>
@@ -4553,21 +4562,21 @@
       </c>
     </row>
     <row r="200">
-      <c r="A200" s="2" t="inlineStr">
+      <c r="A200" s="5" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="B200" s="3" t="n">
+      <c r="B200" s="6" t="n">
         <v>46241</v>
       </c>
-      <c r="C200" s="4" t="n">
+      <c r="C200" s="7" t="n">
         <v>0.7666666666666667</v>
       </c>
-      <c r="D200" s="4" t="n">
+      <c r="D200" s="7" t="n">
         <v>0.7708333333333334</v>
       </c>
-      <c r="E200" s="2" t="inlineStr">
+      <c r="E200" s="5" t="inlineStr">
         <is>
           <t>Night Security</t>
         </is>
@@ -4704,21 +4713,21 @@
       </c>
     </row>
     <row r="207">
-      <c r="A207" s="2" t="inlineStr">
+      <c r="A207" s="5" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="B207" s="3" t="n">
+      <c r="B207" s="6" t="n">
         <v>46248</v>
       </c>
-      <c r="C207" s="4" t="n">
+      <c r="C207" s="7" t="n">
         <v>0.2354166666666667</v>
       </c>
-      <c r="D207" s="4" t="n">
+      <c r="D207" s="7" t="n">
         <v>0.7611111111111111</v>
       </c>
-      <c r="E207" s="2" t="inlineStr">
+      <c r="E207" s="5" t="inlineStr">
         <is>
           <t>Night Security; PLEASE VERIFY: extra punches 05:39 05:39 05:39 05:39 repeated - possible device anomaly</t>
         </is>
@@ -4855,21 +4864,21 @@
       </c>
     </row>
     <row r="214">
-      <c r="A214" s="2" t="inlineStr">
+      <c r="A214" s="5" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="B214" s="3" t="n">
+      <c r="B214" s="6" t="n">
         <v>46255</v>
       </c>
-      <c r="C214" s="4" t="n">
+      <c r="C214" s="7" t="n">
         <v>0.7590277777777777</v>
       </c>
-      <c r="D214" s="4" t="n">
+      <c r="D214" s="7" t="n">
         <v>0.7590277777777777</v>
       </c>
-      <c r="E214" s="2" t="inlineStr">
+      <c r="E214" s="5" t="inlineStr">
         <is>
           <t>Night Security; PLEASE VERIFY: in/out times read identical - likely OCR error</t>
         </is>
@@ -5149,21 +5158,21 @@
       </c>
     </row>
     <row r="229">
-      <c r="A229" s="2" t="inlineStr">
+      <c r="A229" s="5" t="inlineStr">
         <is>
           <t>27</t>
         </is>
       </c>
-      <c r="B229" s="3" t="n">
+      <c r="B229" s="6" t="n">
         <v>46241</v>
       </c>
-      <c r="C229" s="4" t="n">
+      <c r="C229" s="7" t="n">
         <v>0.1486111111111111</v>
       </c>
-      <c r="D229" s="4" t="n">
+      <c r="D229" s="7" t="n">
         <v>0.7201388888888889</v>
       </c>
-      <c r="E229" s="2" t="inlineStr">
+      <c r="E229" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -5296,21 +5305,21 @@
       </c>
     </row>
     <row r="236">
-      <c r="A236" s="2" t="inlineStr">
+      <c r="A236" s="5" t="inlineStr">
         <is>
           <t>27</t>
         </is>
       </c>
-      <c r="B236" s="3" t="n">
+      <c r="B236" s="6" t="n">
         <v>46248</v>
       </c>
-      <c r="C236" s="4" t="n">
+      <c r="C236" s="7" t="n">
         <v>0.2361111111111111</v>
       </c>
-      <c r="D236" s="4" t="n">
+      <c r="D236" s="7" t="n">
         <v>0.7972222222222223</v>
       </c>
-      <c r="E236" s="2" t="inlineStr">
+      <c r="E236" s="5" t="inlineStr">
         <is>
           <t>extra punch: 17:01</t>
         </is>
@@ -5443,21 +5452,21 @@
       </c>
     </row>
     <row r="243">
-      <c r="A243" s="2" t="inlineStr">
+      <c r="A243" s="5" t="inlineStr">
         <is>
           <t>27</t>
         </is>
       </c>
-      <c r="B243" s="3" t="n">
+      <c r="B243" s="6" t="n">
         <v>46255</v>
       </c>
-      <c r="C243" s="4" t="n">
+      <c r="C243" s="7" t="n">
         <v>0.1493055555555556</v>
       </c>
-      <c r="D243" s="4" t="n">
+      <c r="D243" s="7" t="n">
         <v>0.7236111111111111</v>
       </c>
-      <c r="E243" s="2" t="inlineStr">
+      <c r="E243" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -5590,21 +5599,21 @@
       </c>
     </row>
     <row r="250">
-      <c r="A250" s="2" t="inlineStr">
+      <c r="A250" s="5" t="inlineStr">
         <is>
           <t>27</t>
         </is>
       </c>
-      <c r="B250" s="3" t="n">
+      <c r="B250" s="6" t="n">
         <v>46262</v>
       </c>
-      <c r="C250" s="4" t="n">
+      <c r="C250" s="7" t="n">
         <v>0.1493055555555556</v>
       </c>
-      <c r="D250" s="4" t="n">
+      <c r="D250" s="7" t="n">
         <v>0.7159722222222222</v>
       </c>
-      <c r="E250" s="2" t="inlineStr">
+      <c r="E250" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -5741,21 +5750,21 @@
       </c>
     </row>
     <row r="258">
-      <c r="A258" s="2" t="inlineStr">
+      <c r="A258" s="5" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="B258" s="3" t="n">
+      <c r="B258" s="6" t="n">
         <v>46241</v>
       </c>
-      <c r="C258" s="4" t="n">
+      <c r="C258" s="7" t="n">
         <v>0.1791666666666667</v>
       </c>
-      <c r="D258" s="4" t="n">
+      <c r="D258" s="7" t="n">
         <v>0.5618055555555556</v>
       </c>
-      <c r="E258" s="2" t="inlineStr">
+      <c r="E258" s="5" t="inlineStr">
         <is>
           <t>extra punch: 04:18</t>
         </is>
@@ -5888,21 +5897,21 @@
       </c>
     </row>
     <row r="265">
-      <c r="A265" s="2" t="inlineStr">
+      <c r="A265" s="5" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="B265" s="3" t="n">
+      <c r="B265" s="6" t="n">
         <v>46248</v>
       </c>
-      <c r="C265" s="4" t="n">
+      <c r="C265" s="7" t="n">
         <v>0.1743055555555555</v>
       </c>
-      <c r="D265" s="4" t="n">
+      <c r="D265" s="7" t="n">
         <v>0.5298611111111111</v>
       </c>
-      <c r="E265" s="2" t="inlineStr">
+      <c r="E265" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -6035,21 +6044,21 @@
       </c>
     </row>
     <row r="272">
-      <c r="A272" s="2" t="inlineStr">
+      <c r="A272" s="5" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="B272" s="3" t="n">
+      <c r="B272" s="6" t="n">
         <v>46255</v>
       </c>
-      <c r="C272" s="4" t="n">
+      <c r="C272" s="7" t="n">
         <v>0.1854166666666667</v>
       </c>
-      <c r="D272" s="4" t="n">
+      <c r="D272" s="7" t="n">
         <v>0.5319444444444444</v>
       </c>
-      <c r="E272" s="2" t="inlineStr">
+      <c r="E272" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -6182,21 +6191,21 @@
       </c>
     </row>
     <row r="279">
-      <c r="A279" s="2" t="inlineStr">
+      <c r="A279" s="5" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="B279" s="3" t="n">
+      <c r="B279" s="6" t="n">
         <v>46262</v>
       </c>
-      <c r="C279" s="4" t="n">
+      <c r="C279" s="7" t="n">
         <v>0.1881944444444444</v>
       </c>
-      <c r="D279" s="4" t="n">
+      <c r="D279" s="7" t="n">
         <v>0.4055555555555556</v>
       </c>
-      <c r="E279" s="2" t="inlineStr">
+      <c r="E279" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -6973,21 +6982,21 @@
       </c>
     </row>
     <row r="318">
-      <c r="A318" s="2" t="inlineStr">
+      <c r="A318" s="5" t="inlineStr">
         <is>
           <t>34</t>
         </is>
       </c>
-      <c r="B318" s="3" t="n">
+      <c r="B318" s="6" t="n">
         <v>46241</v>
       </c>
-      <c r="C318" s="4" t="n">
+      <c r="C318" s="7" t="n">
         <v>0.1451388888888889</v>
       </c>
-      <c r="D318" s="4" t="n">
+      <c r="D318" s="7" t="n">
         <v>0.7298611111111111</v>
       </c>
-      <c r="E318" s="2" t="inlineStr">
+      <c r="E318" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -7120,21 +7129,21 @@
       </c>
     </row>
     <row r="325">
-      <c r="A325" s="2" t="inlineStr">
+      <c r="A325" s="5" t="inlineStr">
         <is>
           <t>34</t>
         </is>
       </c>
-      <c r="B325" s="3" t="n">
+      <c r="B325" s="6" t="n">
         <v>46248</v>
       </c>
-      <c r="C325" s="4" t="n">
+      <c r="C325" s="7" t="n">
         <v>0.15</v>
       </c>
-      <c r="D325" s="4" t="n">
+      <c r="D325" s="7" t="n">
         <v>0.7076388888888889</v>
       </c>
-      <c r="E325" s="2" t="inlineStr">
+      <c r="E325" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -7267,21 +7276,21 @@
       </c>
     </row>
     <row r="332">
-      <c r="A332" s="2" t="inlineStr">
+      <c r="A332" s="5" t="inlineStr">
         <is>
           <t>34</t>
         </is>
       </c>
-      <c r="B332" s="3" t="n">
+      <c r="B332" s="6" t="n">
         <v>46255</v>
       </c>
-      <c r="C332" s="4" t="n">
+      <c r="C332" s="7" t="n">
         <v>0.275</v>
       </c>
-      <c r="D332" s="4" t="n">
+      <c r="D332" s="7" t="n">
         <v>0.8354166666666667</v>
       </c>
-      <c r="E332" s="2" t="inlineStr">
+      <c r="E332" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -7414,21 +7423,21 @@
       </c>
     </row>
     <row r="339">
-      <c r="A339" s="2" t="inlineStr">
+      <c r="A339" s="5" t="inlineStr">
         <is>
           <t>34</t>
         </is>
       </c>
-      <c r="B339" s="3" t="n">
+      <c r="B339" s="6" t="n">
         <v>46262</v>
       </c>
-      <c r="C339" s="4" t="n">
+      <c r="C339" s="7" t="n">
         <v>0.2805555555555556</v>
       </c>
-      <c r="D339" s="4" t="n">
+      <c r="D339" s="7" t="n">
         <v>0.7701388888888889</v>
       </c>
-      <c r="E339" s="2" t="inlineStr">
+      <c r="E339" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -9066,23 +9075,23 @@
       </c>
     </row>
     <row r="420">
-      <c r="A420" s="2" t="inlineStr">
+      <c r="A420" s="5" t="inlineStr">
         <is>
           <t>39</t>
         </is>
       </c>
-      <c r="B420" s="3" t="n">
+      <c r="B420" s="6" t="n">
         <v>46262</v>
       </c>
-      <c r="C420" s="4" t="n">
+      <c r="C420" s="7" t="n">
         <v>0.25</v>
       </c>
-      <c r="D420" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E420" s="2" t="inlineStr">
+      <c r="D420" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E420" s="5" t="inlineStr">
         <is>
           <t>single punch only</t>
         </is>

</xml_diff>